<commit_message>
Verified inference mode, label cleanup and v2 retrain
- Label cleanup: 97 edits on 67 records (photo artifacts, signatures/dates removed; F3-041 corrected), originals kept as *_v1.jsonl, log in labels/cleanup_log.csv
- train_lora.py: yes/no object questions (--qa) and safe augmentation (--aug)
- autocrop.py: Qwen box around the painted surface, IoU 0.96 vs hand crops
- verify_objects.py: OWLv2 object check calibrated on train (AUC 0.89)
- pipeline.py: rewrite-based check (evaluated, superseded)
- verified.py: three-crop agreement + detector, marks doubtful objects, unclear subjects and background claims
- eval_vlm.py, meaning_charts.py, val_loss.py and charts 9-12
- Validation predictions, manual and object-level reviews, logs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labels/labels.xlsx
+++ b/labels/labels.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P196"/>
+  <dimension ref="A1:Q196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,10 +489,15 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>explanation</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>title_guess</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>palette</t>
         </is>
@@ -556,10 +561,15 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>A single old tree in full autumn color takes over almost the whole picture, so the tree itself becomes the main character. The paint is laid on thick and fast, which makes the leaves feel like they are moving in the wind. Warm orange and ochre against the cool pale sky make the foliage glow. The scene may be read as a celebration of autumn: the last bright moment before the leaves fall.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>Autumn Tree</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>[{"hex": "#b3c9ce", "pct": 23.0}, {"hex": "#6e5642", "pct": 20.0}, {"hex": "#b38046", "pct": 18.2}, {"hex": "#3f332c", "pct": 15.8}, {"hex": "#807770", "pct": 11.7}, {"hex": "#a6a196", "pct": 11.2}]</t>
         </is>
@@ -631,7 +641,12 @@
           <t>high horizon, diagonal hillside, trees scattered in lower half</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>This is a quiet village on a hillside in early spring: brown hills, small houses and a few trees just starting to blossom. The high horizon and the sloping hill pull your eye up through the picture from the trees to the houses. The colors are mostly earthy browns, so the white and pink blossoms stand out as small signs of new life. It may suggest the calm, slow rhythm of country life as the seasons change.</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>[{"hex": "#a37c55", "pct": 31.6}, {"hex": "#7a5744", "pct": 21.4}, {"hex": "#4c3935", "pct": 16.6}, {"hex": "#d2c3b3", "pct": 10.6}, {"hex": "#7b7e77", "pct": 10.6}, {"hex": "#ad998b", "pct": 9.2}]</t>
         </is>
@@ -695,10 +710,15 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>An old stone fortress sits in a green mountain valley, with a river winding toward us in the front. The river works as a path for your eye, leading from the foreground straight to the ruins. The loose, soft brushwork makes the scene feel hazy, like a memory rather than a photograph. Paintings like this often express pride in history and landscape: old walls that have survived among timeless mountains.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Old Fortress by the River</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>[{"hex": "#676b5a", "pct": 20.0}, {"hex": "#878660", "pct": 19.8}, {"hex": "#9c9c7e", "pct": 18.3}, {"hex": "#afb29d", "pct": 17.6}, {"hex": "#525043", "pct": 12.7}, {"hex": "#c8cbbf", "pct": 11.5}]</t>
         </is>
@@ -775,7 +795,12 @@
           <t>central vertical red accent, dark blocks around the edges</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>There is no recognizable subject here; the painting is about color and how it is put on the canvas. Notice the bright red stripe running down the middle, held in place by darker grey and navy blocks on the sides. The patches are layered and loose, so you can follow the movement of the brush. Viewers often read works like this as an emotion, such as tension or warmth breaking through, but there is no single correct meaning.</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>[{"hex": "#8b817d", "pct": 24.6}, {"hex": "#383c3f", "pct": 19.9}, {"hex": "#b57a5a", "pct": 18.7}, {"hex": "#8c6142", "pct": 15.0}, {"hex": "#696968", "pct": 14.2}, {"hex": "#bcaba2", "pct": 7.5}]</t>
         </is>
@@ -847,7 +872,12 @@
           <t>dark mass diagonally from upper center to lower left against light ground</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>There is no recognizable subject here, so the painting is about color, movement and feeling rather than a story. Look at the contrast between the calm, pale area and the dark, stormy cluster of blue, black and red. The thick, scraped paint shows the artist's hand moving quickly. Many viewers read works like this as an emotion or the weather, a storm passing over light, but there is no single correct meaning; part of the point is what you see in it.</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>[{"hex": "#baaa8d", "pct": 24.3}, {"hex": "#918a79", "pct": 22.6}, {"hex": "#696965", "pct": 22.1}, {"hex": "#4b4b4f", "pct": 19.8}, {"hex": "#2a2a2d", "pct": 5.9}, {"hex": "#8d5e47", "pct": 5.4}]</t>
         </is>
@@ -911,10 +941,15 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
+          <t>This abstract painting is built on a contrast: warm pinks and reds on the left meet cold turquoise, blue and black on the right. The muted grey-green border works like a frame inside the frame, focusing attention on that collision. The paint is applied in big sweeping gestures, so the canvas feels energetic. It may be read as a meeting of opposites, warm and cold, calm and dark, without telling any specific story.</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>Warm and Cold</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>[{"hex": "#576261", "pct": 27.0}, {"hex": "#bfbdad", "pct": 15.8}, {"hex": "#bc9581", "pct": 15.2}, {"hex": "#7e8d83", "pct": 15.1}, {"hex": "#a0665f", "pct": 14.2}, {"hex": "#2b353b", "pct": 12.7}]</t>
         </is>
@@ -978,10 +1013,15 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>A bright burst of white and red sits at the center of this square abstract, surrounded by cooler greys and lavenders. Because the strongest colors are in the middle, your eye goes there first and then drifts outward. The layered, overlapping patches give the surface depth and texture. It can be read as an explosion of energy or an emotional center, but the painting invites you to bring your own interpretation.</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
           <t>Composition in Red and Violet</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>[{"hex": "#6e6b70", "pct": 30.3}, {"hex": "#574d53", "pct": 20.8}, {"hex": "#9a8d88", "pct": 17.9}, {"hex": "#965950", "pct": 13.7}, {"hex": "#dad3c9", "pct": 13.5}, {"hex": "#181718", "pct": 3.8}]</t>
         </is>
@@ -1045,10 +1085,15 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
+          <t>A heavy mass of crimson, pink and white paint seems to rise out of a dark grey background, almost like a bouquet or a pile of something alive. The paint is so thick that it looks sculpted, catching light like a relief. The dark surroundings make the warm colors look even more intense. It may suggest flowers, flesh or fire; the artist leaves it open, so the feeling of weight and warmth matters more than the object.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>Red Mass</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>[{"hex": "#6f6862", "pct": 27.8}, {"hex": "#554d4b", "pct": 23.3}, {"hex": "#90564e", "pct": 20.3}, {"hex": "#a5826e", "pct": 16.4}, {"hex": "#c8b19e", "pct": 7.1}, {"hex": "#eaeae4", "pct": 5.1}]</t>
         </is>
@@ -1067,7 +1112,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>A light blue painted field inside a rough white border, with a horizontal row of small colored dots in pink, green, orange, blue and red. Thin black and grey pencil-like lines and scribbles run around and through the dots. The work is behind glass with visible reflections.</t>
+          <t>A light blue painted field inside a rough white border, with a horizontal row of small colored dots in pink, green, orange, blue and red. Thin black and grey pencil-like lines and scribbles run around and through the dots.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1092,7 +1137,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>mixed media on paper, under glass (guess)</t>
+          <t>mixed media on paper (guess)</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1102,7 +1147,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>flat, with glare reflections on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1112,10 +1157,15 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
+          <t>A pale blue field is crossed by a row of small colored dots and light, nervous pencil-like scribbles. The work is very spare: most of the space is left empty so the few marks feel important. The dots can be seen like notes on a line of music, and the scribbles like quick thoughts. It is a playful, light piece that asks you to enjoy simple rhythm and color rather than find a hidden story.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
           <t>Blue Notes</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>[{"hex": "#989992", "pct": 23.6}, {"hex": "#6da2b6", "pct": 22.9}, {"hex": "#b0bdbb", "pct": 19.3}, {"hex": "#498aa1", "pct": 18.9}, {"hex": "#666e6b", "pct": 13.0}, {"hex": "#eaf0ee", "pct": 2.3}]</t>
         </is>
@@ -1134,7 +1184,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>A misty landscape with a single blue tree in the center, standing above a field of grey, rocky texture. The upper part is filled with soft white cloud and grey haze. A signature reading 'Vanni' appears in the lower left; the work is matted and framed behind glass.</t>
+          <t>A misty landscape with a single blue tree in the center, standing above a field of grey, rocky texture. The upper part is filled with soft white cloud and grey haze.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1179,10 +1229,15 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
+          <t>A single blue tree stands alone in a grey, misty landscape, with soft clouds above. Because everything else is pale and blurred, the one blue tree becomes the focus and feels almost unreal. Fog in paintings often creates a mood of silence, distance or dreaming. The picture may be read as an image of solitude, or of something steady and calm surrounded by uncertainty.</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
           <t>Blue Tree in the Mist</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>[{"hex": "#d9d8d2", "pct": 29.6}, {"hex": "#bfbfb7", "pct": 22.8}, {"hex": "#a2a19b", "pct": 18.2}, {"hex": "#858079", "pct": 16.1}, {"hex": "#605e5d", "pct": 9.5}, {"hex": "#567c9c", "pct": 3.7}]</t>
         </is>
@@ -1201,7 +1256,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>An abstract work with vertical streaks and scraped layers of red, pink, ochre, gold and white over a pale blue ground. The surface looks scraped and dripped, revealing underlayers. Strong reflections of a window and room are visible on the glass.</t>
+          <t>An abstract work with vertical streaks and scraped layers of red, pink, ochre, gold and white over a pale blue ground. The surface looks scraped and dripped, revealing underlayers.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1236,7 +1291,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>flat, with strong glare reflections on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1246,10 +1301,15 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
+          <t>Streaks of red, pink, gold and white run down over a pale blue ground, as if the paint has been dragged and scraped. Scraping lets older layers show through, so the surface feels like it has a history. The vertical movement can remind viewers of rain, dripping light or a curtain of color. It is an abstract work about texture and energy.</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
           <t>Red Rain</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>[{"hex": "#a9adad", "pct": 23.3}, {"hex": "#a18777", "pct": 21.3}, {"hex": "#7a634e", "pct": 19.5}, {"hex": "#dad8d4", "pct": 16.5}, {"hex": "#43322b", "pct": 10.5}, {"hex": "#9b3439", "pct": 8.9}]</t>
         </is>
@@ -1313,10 +1373,15 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
+          <t>A fluffy white creature in a pointed hat sits at a little café table holding a cup, under an awning that reads 'CAFE'. Everything is painted in soft, misty blue, which gives the scene a calm, dreamy, slightly rainy mood. The creature looks like a character from a fairy tale or children's book. It may be read as a gentle picture of enjoying a quiet moment alone, treated with humor and warmth.</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
           <t>Café in the Rain</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>[{"hex": "#aabcba", "pct": 23.4}, {"hex": "#8ea7ab", "pct": 23.0}, {"hex": "#7c979b", "pct": 20.5}, {"hex": "#678286", "pct": 18.5}, {"hex": "#cdd3ce", "pct": 10.7}, {"hex": "#59594f", "pct": 4.0}]</t>
         </is>
@@ -1380,10 +1445,15 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
+          <t>This is the inside of a café or dining hall, painted almost only in greys, whites and browns. Light comes in through tall windows at the back, so the tables and the seated figure appear partly as silhouettes. The quick, loose brushwork captures the atmosphere more than the details, the way you remember a place rather than how it exactly looked. The muted colors give it a quiet, slightly lonely mood.</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
           <t>In the Café</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>[{"hex": "#a9a49b", "pct": 27.4}, {"hex": "#93908b", "pct": 27.3}, {"hex": "#c3beb3", "pct": 17.6}, {"hex": "#7a7875", "pct": 16.6}, {"hex": "#e5e3d8", "pct": 7.5}, {"hex": "#4e4d4a", "pct": 3.6}]</t>
         </is>
@@ -1447,10 +1517,15 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
+          <t>A humorous scene in a café: a grumpy man holds dominoes, a woman in a hat leans on him, another man hides behind his newspaper, and a waiter looms behind them. The exaggerated faces and bodies are caricature, a style that makes fun of everyday people to show their personalities. The single bulb hanging over the table works like a spotlight, as if we're watching a small stage play. It may be read as a gentle joke about café life, where everyone is together but each person is in their own world.</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
           <t>Dominoes at the Café</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>[{"hex": "#7e4a22", "pct": 32.0}, {"hex": "#282526", "pct": 21.7}, {"hex": "#aa7837", "pct": 21.6}, {"hex": "#4c4844", "pct": 9.7}, {"hex": "#9f8e76", "pct": 8.9}, {"hex": "#c6bca5", "pct": 6.0}]</t>
         </is>
@@ -1514,10 +1589,15 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
+          <t>Chairs and tables tilt and tumble across the canvas, drawn with thick black outlines over flat yellow, ochre and grey shapes. Showing objects from several angles at once is a cubist idea: instead of one viewpoint, you see how the object might look as you move around it. With only a small wine glass and no people, the café feels empty. It may suggest the end of the evening, or a memory of a place spinning a little.</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
           <t>Empty Café</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>[{"hex": "#343138", "pct": 24.5}, {"hex": "#c8b08c", "pct": 22.6}, {"hex": "#8d857c", "pct": 16.6}, {"hex": "#c99c4e", "pct": 14.9}, {"hex": "#5d5858", "pct": 11.4}, {"hex": "#d9d1c5", "pct": 9.9}]</t>
         </is>
@@ -1536,7 +1616,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>A collage-like composition of elegant figures in long coats, hats and gowns arranged across red, blue, grey and white color blocks. Handwritten text fragments, a red plant and a blue X shape appear among the figures. The work is framed behind glass with visible reflections.</t>
+          <t>A collage-like composition of elegant figures in long coats, hats and gowns arranged across red, blue, grey and white color blocks. Handwritten text fragments, a red plant and a blue X shape appear among the figures.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1571,7 +1651,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>flat, with reflections on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1581,10 +1661,15 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
+          <t>Elegant figures in long coats, hats and gowns are arranged across blocks of red, blue, grey and white, together with handwritten text and a red plant. The mix of figures, writing and flat color areas makes it feel like a collage or a page from a fashion scrapbook. The clothes suggest an older era. The work may be read as a nostalgic look at style and society, where people are shown almost like characters on display.</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
           <t>Promenade</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>[{"hex": "#837775", "pct": 24.1}, {"hex": "#b49693", "pct": 22.5}, {"hex": "#c9716c", "pct": 20.5}, {"hex": "#c1bdbb", "pct": 13.3}, {"hex": "#5485b8", "pct": 10.1}, {"hex": "#593e3d", "pct": 9.5}]</t>
         </is>
@@ -1603,7 +1688,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Same artwork as F1-016, photographed again: elegant figures in coats, hats and gowns over red, blue, grey and white color blocks, with handwritten text fragments, a red plant and a blue X. Reflections on the glass are visible in the lower center.</t>
+          <t>Elegant figures in coats, hats and gowns over red, blue, grey and white color blocks, with handwritten text fragments, a red plant and a blue X.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1638,7 +1723,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>flat, with reflections on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1648,10 +1733,15 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
+          <t>Elegant figures in long coats, hats and gowns are arranged across blocks of red, blue, grey and white, together with handwritten text and a red plant. The mix of figures, writing and flat color areas makes it feel like a collage or a page from a fashion scrapbook. The clothes suggest an older era. The work may be read as a nostalgic look at style and society, where people are shown almost like characters on display.</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
           <t>Promenade</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>[{"hex": "#c87875", "pct": 24.5}, {"hex": "#837674", "pct": 21.2}, {"hex": "#aea2a1", "pct": 20.3}, {"hex": "#d0ccca", "pct": 16.0}, {"hex": "#5687ba", "pct": 9.0}, {"hex": "#583b3c", "pct": 9.0}]</t>
         </is>
@@ -1715,10 +1805,15 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
+          <t>The front of a building, perhaps a café since a sign reads '...CAFE', is broken down into big vertical panels of green, white and blue. White grid lines look like scaffolding or window frames. The paint is scraped and worn, so the facade looks weathered, like an old city wall. It may be read as a portrait of a city corner, simplified until it becomes almost an abstract pattern.</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
           <t>Café Facade</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>[{"hex": "#505b54", "pct": 21.5}, {"hex": "#353d37", "pct": 18.0}, {"hex": "#d3cfcc", "pct": 16.9}, {"hex": "#b3b8b9", "pct": 15.1}, {"hex": "#6e7875", "pct": 15.0}, {"hex": "#899ca6", "pct": 13.5}]</t>
         </is>
@@ -1782,10 +1877,15 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
+          <t>Tall buildings with arched windows, a dome and a spire rise up through drips and scraped paint, as if the city is melting or appearing out of fog. The muted blues, ochres and rust tones make it feel old and faded. Instead of drawing every detail, the artist suggests the buildings, so we fill in the rest from memory. It may be read as a dream or memory of an old town rather than a real view.</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
           <t>Old Town</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>[{"hex": "#8e897d", "pct": 26.4}, {"hex": "#746d63", "pct": 24.9}, {"hex": "#97a4a3", "pct": 16.7}, {"hex": "#5c4e42", "pct": 15.5}, {"hex": "#2c2624", "pct": 10.1}, {"hex": "#c4b7a0", "pct": 6.4}]</t>
         </is>
@@ -1804,7 +1904,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>A densely detailed fantasy scene on a black background, filled with floating figures, masks, flowers, swirling ornaments and patterned shapes. A white round object sits near the center and a jester-like figure appears in the lower right. Initials and '24' are written in the lower left; the work is in a gold frame behind glass.</t>
+          <t>A densely detailed fantasy scene on a black background, filled with floating figures, masks, flowers, swirling ornaments and patterned shapes. A white round object sits near the center and a jester-like figure appears in the lower right.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1849,10 +1949,15 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
+          <t>A crowded fantasy world on a black background: floating figures, masks, flowers, swirls and patterns fill every corner. A white round shape near the center acts like a moon or a stage light, and a jester-like figure appears in the lower right. The dense, decorative style invites you to look closely and keep discovering new details. It may be read as a carnival or a dream where real and imaginary characters mix.</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
           <t>Carnival of Dreams</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>[{"hex": "#74706c", "pct": 25.8}, {"hex": "#5d534c", "pct": 24.9}, {"hex": "#8c8e8d", "pct": 21.1}, {"hex": "#c7b090", "pct": 9.9}, {"hex": "#3a322f", "pct": 9.7}, {"hex": "#a97561", "pct": 8.5}]</t>
         </is>
@@ -1916,10 +2021,15 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
+          <t>A woman with short black hair sits with her legs crossed, holding a tall colorful drink. The background is broken into loose patches of yellow, pink and blue rather than showing a real room, so all attention is on her pose and expression. Her pale face and calm look feel thoughtful, maybe a little distant. It can be read as a portrait of a modern woman taking a quiet moment for herself.</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
           <t>Woman with a Drink</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>[{"hex": "#232223", "pct": 28.0}, {"hex": "#c4ac8d", "pct": 27.1}, {"hex": "#6e6e75", "pct": 24.4}, {"hex": "#7c96ac", "pct": 8.8}, {"hex": "#d9a32a", "pct": 8.2}, {"hex": "#b23620", "pct": 3.5}]</t>
         </is>
@@ -1983,10 +2093,15 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
+          <t>Instead of faces, the painting shows only legs and shoes under office desks: pinstriped trousers and heels on one side, bare legs and loafers on the other. Cutting the picture at knee height is a clever choice, because shoes and posture alone tell us about the people. It feels like a hidden view of office life that we normally don't notice. It may be read as a playful comment on work, routine and the little gestures people make when they think no one is looking.</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
           <t>Under the Desk</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>[{"hex": "#a69b8a", "pct": 30.0}, {"hex": "#beb5a9", "pct": 17.5}, {"hex": "#433c39", "pct": 13.9}, {"hex": "#241d1d", "pct": 13.4}, {"hex": "#877e72", "pct": 13.2}, {"hex": "#66594e", "pct": 11.9}]</t>
         </is>
@@ -2050,10 +2165,15 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
+          <t>Two heads with big round eyes peek up at each other from a field of fluffy red flowers. The faces are drawn with quick, simple black lines, which gives them a cartoon-like charm. Their pursed lips and close faces suggest a kiss, a secret or a flirt. The bright red flowers below may stand for love or passion, making it a playful, tender picture of two people being close.</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
           <t>Two in the Flowers</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>[{"hex": "#9c1021", "pct": 42.1}, {"hex": "#cdc2bc", "pct": 28.1}, {"hex": "#b73746", "pct": 15.5}, {"hex": "#c4757a", "pct": 9.4}, {"hex": "#211717", "pct": 2.7}, {"hex": "#70645e", "pct": 2.3}]</t>
         </is>
@@ -2087,7 +2207,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>A vineyard landscape with rows of dark vine stems on bright green rolling slopes in the foreground. A large flat-topped khaki and brown mountain rises behind, under a pale olive sky. A signature is visible in the lower right.</t>
+          <t>A vineyard landscape with rows of dark vine stems on bright green rolling slopes in the foreground. A large flat-topped khaki and brown mountain rises behind, under a pale olive sky.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2130,7 +2250,12 @@
           <t>green foreground slopes, mountain band across the middle, high horizon</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Rows of dark vines stand on bright green hills in front of a big flat-topped mountain. The landscape is simplified into broad color areas, which makes it calm and easy to read. Vineyards are an important part of many cultures, so the scene can be seen as a portrait of land, work and tradition. The pale sky and soft colors give it a peaceful mood.</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>[{"hex": "#807a2c", "pct": 29.9}, {"hex": "#968940", "pct": 23.5}, {"hex": "#666622", "pct": 20.6}, {"hex": "#a7935a", "pct": 20.4}, {"hex": "#3d3919", "pct": 5.0}, {"hex": "#cdc1b4", "pct": 0.5}]</t>
         </is>
@@ -2207,7 +2332,12 @@
           <t>wide sky in upper two thirds, dark forms along the bottom</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>A soft pink and blue evening sky sits above a dark line of trees or bushes. The colors run into each other like watercolor, so the shapes are blurred and gentle. Most of the picture is sky, which makes the land feel small and quiet. It may be read as a simple moment at dusk, when the light fades and everything becomes still.</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>[{"hex": "#ac8e79", "pct": 32.0}, {"hex": "#b3a79b", "pct": 18.8}, {"hex": "#9a9896", "pct": 18.2}, {"hex": "#21241e", "pct": 12.9}, {"hex": "#3b4538", "pct": 12.7}, {"hex": "#6d6758", "pct": 5.3}]</t>
         </is>
@@ -2271,10 +2401,15 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
+          <t>Two round, smiling angels with golden halos stand together holding a plate of red eggs and a cake with a candle. Red-dyed eggs are a well-known Easter tradition in Orthodox Christian countries, so the painting celebrates that holiday. The simple, childlike drawing style makes the scene cheerful and friendly rather than serious. It is a warm picture about celebration, faith and sharing.</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
           <t>Easter Angels</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>[{"hex": "#c6ad8f", "pct": 34.6}, {"hex": "#76837b", "pct": 17.8}, {"hex": "#4b5c7d", "pct": 14.5}, {"hex": "#b1946e", "pct": 13.4}, {"hex": "#ad5625", "pct": 10.2}, {"hex": "#465a46", "pct": 9.5}]</t>
         </is>
@@ -2293,7 +2428,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>A small angel in a long blue robe with white wings and golden hair is painted on a dark bird feather, mounted on a white board. The angel holds a golden panpipe-like instrument and stands on grey rocks. 'Puerto Rico' is written in the upper left and a signature with '2023' in the lower right.</t>
+          <t>A small angel in a long blue robe with white wings and golden hair is painted on a dark bird feather, mounted on a white board. The angel holds a golden panpipe-like instrument and stands on grey rocks. 'Puerto Rico' is written in the upper left.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2328,7 +2463,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>flat, with shadow of photographer on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2338,10 +2473,15 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
+          <t>A tiny angel with white wings and a blue robe is painted directly onto a dark bird feather. Painting on such an unusual, delicate surface is a special craft and makes the angel seem light, as if it could float away. The angel plays a golden wind instrument, a common image of heavenly music. The words 'Puerto Rico' written on the board suggest a place connected to the work.</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
           <t>Angel on a Feather</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t>[{"hex": "#b9a8a0", "pct": 38.7}, {"hex": "#a7948c", "pct": 34.2}, {"hex": "#372c2f", "pct": 11.6}, {"hex": "#644e41", "pct": 6.3}, {"hex": "#7c7679", "pct": 5.4}, {"hex": "#38527f", "pct": 3.8}]</t>
         </is>
@@ -2418,7 +2558,12 @@
           <t>all-over diagonal strokes with darker center</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bright yellow strokes slash diagonally across darker blacks, greys and blues, creating a strong sense of speed. Diagonal lines in art usually feel more active than horizontal or vertical ones. The paint is thick and smeared, so you can almost feel the force of the brush. It may be read as lightning, movement or a burst of energy, but it is mainly about action and emotion rather than a subject.</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
         <is>
           <t>[{"hex": "#685f55", "pct": 23.6}, {"hex": "#9d7f48", "pct": 18.8}, {"hex": "#978b83", "pct": 17.1}, {"hex": "#d5b430", "pct": 16.1}, {"hex": "#393431", "pct": 15.1}, {"hex": "#d1c1b0", "pct": 9.3}]</t>
         </is>
@@ -2495,7 +2640,12 @@
           <t>central triangular shape surrounded by all-over splatter</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>A big yellow-green triangle rises in the center like a mountain, surrounded by splashes and drips of white, red, black, teal and purple. Dripping and flicking paint onto the canvas is a technique that lets chance and movement shape the picture. The calm triangle in the middle contrasts with the wild splatter around it. It may be read as a mountain in a storm, or simply as order in the middle of chaos.</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>[{"hex": "#d2cbbf", "pct": 25.1}, {"hex": "#ac9687", "pct": 19.5}, {"hex": "#a58b38", "pct": 16.4}, {"hex": "#5c6250", "pct": 15.1}, {"hex": "#272824", "pct": 13.4}, {"hex": "#923430", "pct": 10.5}]</t>
         </is>
@@ -2529,7 +2679,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>A grey smoky field with soot-like dark patches and layered translucent paper shapes. Thin red curving lines loop across the surface like a maze. A small signature appears in the lower right.</t>
+          <t>A grey smoky field with soot-like dark patches and layered translucent paper shapes. Thin red curving lines loop across the surface like a maze.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2572,7 +2722,12 @@
           <t>all-over texture with looping lines across the vertical field</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>A smoky grey surface with soot-like stains is crossed by thin red lines that loop like a maze. The layered, translucent shapes make it feel like looking through fog or old paper. The red lines stand out as the only strong color, like a path or a thread you could follow. It may be read as a labyrinth of thoughts or memories, where the way forward is hidden.</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>[{"hex": "#918b81", "pct": 25.7}, {"hex": "#7d756b", "pct": 22.9}, {"hex": "#a5a298", "pct": 20.2}, {"hex": "#645c51", "pct": 14.7}, {"hex": "#c1bdb4", "pct": 9.9}, {"hex": "#413a31", "pct": 6.7}]</t>
         </is>
@@ -2606,7 +2761,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Two stylized female faces with long multicolored streaked hair, red cheeks and red lips lean toward each other on a grey-green background. They are drawn in pastel-like lines in blue, pink, green and white. A signature 'Tekla Mela...' is in the lower right; the photographer is reflected in the glass.</t>
+          <t>Two stylized female faces with long multicolored streaked hair, red cheeks and red lips lean toward each other on a grey-green background. They are drawn in pastel-like lines in blue, pink, green and white.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2641,7 +2796,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>flat, with reflections on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2649,7 +2804,12 @@
           <t>two faces side by side filling the horizontal frame</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Two women with long, multicolored hair and red cheeks lean their heads close together. The way they turn toward each other suggests whispering, sharing a secret or gossiping. They are drawn with colorful pastel lines rather than filled-in shapes, which keeps the image light and lively. It can be read as a playful picture of friendship and of the small private conversations people share.</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>[{"hex": "#858275", "pct": 31.2}, {"hex": "#7b786b", "pct": 24.6}, {"hex": "#8f8d82", "pct": 23.9}, {"hex": "#9b9a91", "pct": 15.4}, {"hex": "#656250", "pct": 4.2}, {"hex": "#efe0d1", "pct": 0.7}]</t>
         </is>
@@ -2726,7 +2886,12 @@
           <t>figures low left, carriage low right, tree upper center</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Three veiled figures sit on a red carpet facing an empty golden carriage, with a single pink tree behind them on a pink background. The scene is flat and strange, like a dream where the rules of real life don't apply. The empty carriage makes us ask who it is waiting for, or who has left. It may be read as a scene about ritual, waiting or a journey that hasn't started yet.</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>[{"hex": "#ba7297", "pct": 39.2}, {"hex": "#c58aa7", "pct": 35.6}, {"hex": "#a24c77", "pct": 13.3}, {"hex": "#72382c", "pct": 5.1}, {"hex": "#231410", "pct": 4.9}, {"hex": "#c9beb5", "pct": 1.7}]</t>
         </is>
@@ -2760,7 +2925,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>A still life of a dark green bottle and a large olive-colored two-handled jug, with three red pomegranates in front on a crumpled white cloth. A pale green and pink drapery hangs behind. There are reflections on the glass.</t>
+          <t>A still life of a dark green bottle and a large olive-colored two-handled jug, with three red pomegranates in front on a crumpled white cloth. A pale green and pink drapery hangs behind.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2803,7 +2968,12 @@
           <t>jug center, bottle left, fruit row along the lower middle</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>A classic still life: a dark green bottle, a large jug and three red pomegranates on a crumpled white cloth. Still lifes let artists practice light, shape and texture, like the shine of glass or the folds of fabric. Pomegranates are a strong symbol in many cultures, often linked to life and abundance. The calm arrangement invites you to slow down and look at everyday objects carefully.</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>[{"hex": "#cebeac", "pct": 22.1}, {"hex": "#706a5f", "pct": 19.0}, {"hex": "#b69e8d", "pct": 17.1}, {"hex": "#897e73", "pct": 15.9}, {"hex": "#949e8e", "pct": 14.5}, {"hex": "#55443e", "pct": 11.4}]</t>
         </is>
@@ -2880,7 +3050,12 @@
           <t>one-point perspective toward the café sign, figures along both sides</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>A violet night street leads toward a glowing 'Cafe' sign, with tall buildings lit by small yellow windows. Small doll-like women in short dresses and boots stand along both sides. The perspective pulls your eye straight down the street to the café, like walking into the night. The strong purple color and the figures suggest city nightlife, possibly with a slightly ironic or critical tone.</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
         <is>
           <t>[{"hex": "#987abf", "pct": 33.3}, {"hex": "#7f63af", "pct": 31.9}, {"hex": "#624e94", "pct": 19.8}, {"hex": "#473d63", "pct": 6.9}, {"hex": "#c5b9c9", "pct": 6.4}, {"hex": "#cdb872", "pct": 1.7}]</t>
         </is>
@@ -2957,7 +3132,12 @@
           <t>tables in foreground and middle ground, building in distance under trees</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>People dressed in old-fashioned clothes sit at round tables in an outdoor park café, with bottles and glasses on the tables and a white building with a 'CAFE' sign behind the trees. The simple, slightly naive drawing style makes the scene charming rather than realistic. It looks back at an earlier time when cafés were places to see and be seen. The grey sky adds a soft, nostalgic mood.</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
         <is>
           <t>[{"hex": "#463a37", "pct": 26.1}, {"hex": "#675850", "pct": 21.1}, {"hex": "#89796e", "pct": 17.5}, {"hex": "#2a201f", "pct": 16.4}, {"hex": "#ad9c8a", "pct": 11.6}, {"hex": "#d3c5b2", "pct": 7.2}]</t>
         </is>
@@ -2991,7 +3171,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Same artwork as F1-040, photographed again: a dark green bottle and an olive two-handled jug with three red pomegranates on a crumpled white cloth, against green and pink drapery. Reflections on the glass are visible.</t>
+          <t>A dark green bottle and an olive two-handled jug with three red pomegranates on a crumpled white cloth, against green and pink drapery.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3034,7 +3214,12 @@
           <t>jug center, bottle left, fruit row along the lower middle</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>A classic still life: a dark green bottle, a large jug and three red pomegranates on a crumpled white cloth. Still lifes let artists practice light, shape and texture, like the shine of glass or the folds of fabric. Pomegranates are a strong symbol in many cultures, often linked to life and abundance. The calm arrangement invites you to slow down and look at everyday objects carefully.</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
         <is>
           <t>[{"hex": "#706e62", "pct": 24.4}, {"hex": "#cfbeac", "pct": 19.1}, {"hex": "#b5a18e", "pct": 18.6}, {"hex": "#8c9686", "pct": 15.5}, {"hex": "#564841", "pct": 12.1}, {"hex": "#997a6b", "pct": 10.4}]</t>
         </is>
@@ -3111,7 +3296,12 @@
           <t>concentric frames receding toward the lower left</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Rectangles inside rectangles, in pink, orange, blue, green and black, fill the canvas, decorated with tiny squares, spirals and lines. The nested frames create a sense of depth, like looking down a tunnel or through layers of windows. A red scribbled circle and thin black drips break the tidy pattern. It may be read as a game between order and disorder, or simply enjoyed as a rich, rhythmic design.</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
         <is>
           <t>[{"hex": "#32373b", "pct": 23.6}, {"hex": "#557355", "pct": 21.0}, {"hex": "#436487", "pct": 15.3}, {"hex": "#db8b23", "pct": 14.9}, {"hex": "#994a47", "pct": 14.7}, {"hex": "#9a7d7f", "pct": 10.6}]</t>
         </is>
@@ -3130,7 +3320,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Three blue-violet irises with yellow beards and green stems stand against a golden ochre background. Thick impasto gives the petals a sculpted texture. Initials 'A.T.' and '2016' are written in the lower right.</t>
+          <t>Three blue-violet irises with yellow beards and green stems stand against a golden ochre background. Thick impasto gives the petals a sculpted texture.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3175,10 +3365,15 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
+          <t>Three blue-violet irises stand against a warm golden background. The paint on the petals is so thick that the flowers almost stand out from the canvas. Blue and gold are opposite colors, so they make each other look brighter. Irises are often linked with spring, hope and beauty, and the picture is a simple celebration of flowers.</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
           <t>Irises</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
+      <c r="Q39" t="inlineStr">
         <is>
           <t>[{"hex": "#bc8d39", "pct": 22.9}, {"hex": "#525978", "pct": 19.1}, {"hex": "#8e632c", "pct": 18.3}, {"hex": "#c6a66d", "pct": 16.5}, {"hex": "#7783a6", "pct": 12.4}, {"hex": "#403838", "pct": 10.7}]</t>
         </is>
@@ -3197,7 +3392,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>A woven or embroidered tapestry-like image of a bright interior with white curtains and a vase of pink and dark flowers in the lower left. Soft lilac, cream and grey tones dominate, and the stitched texture is visible. Reflections of ceiling lights appear on the glass.</t>
+          <t>A woven or embroidered tapestry-like image of a bright interior with white curtains and a vase of pink and dark flowers in the lower left. Soft lilac, cream and grey tones dominate, and the stitched texture is visible.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3242,10 +3437,15 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
+          <t>This image is made of thread or fabric rather than paint: a bright room with white curtains and a vase of flowers near the window. Textile art takes a lot of patience, and the stitched texture gives the light a soft, woven quality. The pale lilac and cream colors make the room feel airy and peaceful. It may be read as a quiet moment of daylight at home.</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
           <t>Flowers at the Window</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="Q40" t="inlineStr">
         <is>
           <t>[{"hex": "#a99d8e", "pct": 22.9}, {"hex": "#928579", "pct": 22.0}, {"hex": "#7d6b5f", "pct": 21.1}, {"hex": "#bfb6a6", "pct": 15.0}, {"hex": "#5b4c4b", "pct": 11.6}, {"hex": "#2d2625", "pct": 7.3}]</t>
         </is>
@@ -3264,7 +3464,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>A tapestry-like landscape of a village with small white and pink houses among purple, orange and red flowering trees. Green and lilac hills rise behind under a blue and white sky. The stitched texture is visible, with light reflections on the glass.</t>
+          <t>A tapestry-like landscape of a village with small white and pink houses among purple, orange and red flowering trees. Green and lilac hills rise behind under a blue and white sky. The stitched texture is visible.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3309,10 +3509,15 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
+          <t>A small village with white and pink houses sits among trees blooming in purple, orange and red, with green hills behind. It is made with thread or fabric, so the colors are built up stitch by stitch. The bright blossoms and blue sky give it a cheerful spring mood. It may be read as an idealized, happy picture of village life in bloom.</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
           <t>Village in Spring</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="Q41" t="inlineStr">
         <is>
           <t>[{"hex": "#8b7f7e", "pct": 23.1}, {"hex": "#b5b3aa", "pct": 20.7}, {"hex": "#aa9684", "pct": 20.6}, {"hex": "#6f6a5c", "pct": 13.9}, {"hex": "#98694d", "pct": 11.0}, {"hex": "#5b3a38", "pct": 10.8}]</t>
         </is>
@@ -3331,7 +3536,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>A stylized female figure with a faceless pale oval head and flowing auburn hair, wearing a long rust-red dress that sweeps diagonally across the canvas. The background is cream and ochre with soft brown shadows. A signature 'B' with '2010' appears in the lower right.</t>
+          <t>A stylized female figure with a faceless pale oval head and flowing auburn hair, wearing a long rust-red dress that sweeps diagonally across the canvas. The background is cream and ochre with soft brown shadows.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3376,10 +3581,15 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
+          <t>A woman with flowing auburn hair and a long rust-red dress sweeps diagonally across the canvas, but her face is left blank. Leaving out the face turns her into a symbol rather than a specific person, so we focus on her movement and elegance. The diagonal pose and the curve of the dress create a feeling of motion, like dancing or walking in the wind. It may be read as a picture of femininity and grace.</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
           <t>Woman in Red</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
+      <c r="Q42" t="inlineStr">
         <is>
           <t>[{"hex": "#c8c1ae", "pct": 28.3}, {"hex": "#beab8b", "pct": 22.7}, {"hex": "#965038", "pct": 16.5}, {"hex": "#70362c", "pct": 14.3}, {"hex": "#b58d60", "pct": 12.0}, {"hex": "#47231d", "pct": 6.2}]</t>
         </is>
@@ -3398,7 +3608,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>A field of red, orange and yellow flowers under a blue sky, covered with dense splatters and drips of white, yellow and orange paint. Green stems fill the lower part. The work is behind glass with a window reflection.</t>
+          <t>A field of red, orange and yellow flowers under a blue sky, covered with dense splatters and drips of white, yellow and orange paint. Green stems fill the lower part.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3433,7 +3643,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>bright, flat, with reflections on glass</t>
+          <t>bright, flat</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3443,10 +3653,15 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
+          <t>A meadow of red, orange and yellow flowers sits under a blue sky, covered with splashes and drips of paint. The flicked and dripped paint makes the flowers feel alive and moving, as if the wind or the sun is shaking them. The artist cares more about energy and color than exact flower shapes. It is a joyful picture that may express the excitement of summer.</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
           <t>Wild Meadow</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>[{"hex": "#657274", "pct": 36.3}, {"hex": "#525242", "pct": 22.7}, {"hex": "#a57849", "pct": 12.8}, {"hex": "#894b33", "pct": 12.6}, {"hex": "#a3978c", "pct": 12.5}, {"hex": "#dad3cd", "pct": 3.2}]</t>
         </is>
@@ -3510,10 +3725,15 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
+          <t>A pale, thin figure with a visible spine stands in profile with a hammer stuck in its head, while a red heart sits outside its body inside a white outline. This is surrealism: impossible, dreamlike images used to show feelings. The hammer may stand for pain, pressure or a thought that hurts, and the separated heart for emotions cut off from the body. Dark green and bare black branches make the mood heavy and unsettling.</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
           <t>Hammer and Heart</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
+      <c r="Q44" t="inlineStr">
         <is>
           <t>[{"hex": "#282928", "pct": 39.3}, {"hex": "#354a37", "pct": 29.1}, {"hex": "#cbc2c1", "pct": 14.3}, {"hex": "#8b6f5c", "pct": 6.5}, {"hex": "#ad9897", "pct": 6.0}, {"hex": "#793738", "pct": 4.8}]</t>
         </is>
@@ -3532,7 +3752,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>A lively ballroom or festive scene with women in long red, pink and white gowns dancing beneath hanging garlands and streamers. The strokes are loose and expressive in yellow, pink, green and white. A signature appears in the lower left; the work is matted behind glass.</t>
+          <t>A lively ballroom or festive scene with women in long red, pink and white gowns dancing beneath hanging garlands and streamers. The strokes are loose and expressive in yellow, pink, green and white.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3577,10 +3797,15 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
+          <t>Women in long red, pink and white gowns dance under garlands and streamers, painted with quick, loose strokes. The fast brushwork captures movement and the feeling of a party rather than precise details. Warm pinks and yellows make the scene glow like festive lights. It may be read as a celebration, a ball or a happy memory of music and dancing.</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
           <t>The Ball</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr">
+      <c r="Q45" t="inlineStr">
         <is>
           <t>[{"hex": "#b6b2a3", "pct": 28.8}, {"hex": "#a89987", "pct": 24.3}, {"hex": "#cbc8b8", "pct": 17.3}, {"hex": "#877e61", "pct": 13.1}, {"hex": "#744541", "pct": 8.8}, {"hex": "#b3ab5b", "pct": 7.7}]</t>
         </is>
@@ -3599,7 +3824,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>A calligraphic artwork in which black Arabic script forms the shape of a whirling dervish with a tall hat and flared skirt. Small red ornamented shapes mark the hat, a foot and a decorative medallion on the left. The ground is pale marbled cream, matted inside a dark frame.</t>
+          <t>A calligraphic artwork in which black Arabic script forms the shape of a whirling dervish with a tall hat and flared skirt. Small red ornamented shapes mark the hat, a foot and a decorative medallion on the left. The ground is pale marbled cream.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3644,10 +3869,15 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
+          <t>Here the picture is made of writing: black Arabic calligraphy forms the shape of a whirling dervish, a dancer with a tall hat and wide skirt. Whirling is a spiritual practice in Sufism, a mystical tradition in Islam, where spinning is a form of prayer and meditation. In Islamic art, beautiful writing is a high art form, so combining words and a dancing figure joins text and devotion. Small red ornaments add rhythm and accent.</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
           <t>Whirling Dervish</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="Q46" t="inlineStr">
         <is>
           <t>[{"hex": "#c1baac", "pct": 40.6}, {"hex": "#d2cfc4", "pct": 22.2}, {"hex": "#aba499", "pct": 16.1}, {"hex": "#847e79", "pct": 7.5}, {"hex": "#5e5152", "pct": 6.9}, {"hex": "#29272d", "pct": 6.7}]</t>
         </is>
@@ -3724,7 +3954,12 @@
           <t>central standing figure flanked symmetrically by two seated figures</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Three nude women, one seen from behind and two seated, are shown in soft cream and beige, with small sailboats on the sea behind them. The raised outlines make the painting look almost like a carved relief. The calm, single color gives the scene a timeless, classical feel, like an ancient wall decoration. It may be read as a peaceful image of the human body, nature and the sea.</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
         <is>
           <t>[{"hex": "#b5ada1", "pct": 26.0}, {"hex": "#d0cec5", "pct": 24.7}, {"hex": "#c2bdb2", "pct": 23.7}, {"hex": "#a69b8e", "pct": 16.7}, {"hex": "#948574", "pct": 7.8}, {"hex": "#574e43", "pct": 1.1}]</t>
         </is>
@@ -3743,7 +3978,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>A nude female figure with arms raised above her head appears to rise out of a large red hibiscus flower on the left. The canvas is filled with oversized red and orange hibiscus blossoms, opening onto a glowing yellow and turquoise space in the center. A signature is in the lower right.</t>
+          <t>A nude female figure with arms raised above her head appears to rise out of a large red hibiscus flower on the left. The canvas is filled with oversized red and orange hibiscus blossoms, opening onto a glowing yellow and turquoise space in the center.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3788,10 +4023,15 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
+          <t>A nude woman with raised arms seems to grow out of a giant red hibiscus flower, surrounded by more huge blossoms opening onto a glowing center. Mixing a human body with a flower is a way to connect women, beauty and nature. The oversized flowers and hot colors make the scene feel sensual and full of energy. It may be read as a celebration of femininity and life blooming.</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
           <t>Flower Woman</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="Q48" t="inlineStr">
         <is>
           <t>[{"hex": "#7e2d39", "pct": 32.6}, {"hex": "#974045", "pct": 31.6}, {"hex": "#a17053", "pct": 15.7}, {"hex": "#ae9c7a", "pct": 12.4}, {"hex": "#7ab9bc", "pct": 4.2}, {"hex": "#2c3b3d", "pct": 3.5}]</t>
         </is>
@@ -3810,7 +4050,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Same artwork as F1-056, photographed again: a pale ribbed surreal figure in profile with a hammer in its head and a red anatomical heart outside the body inside a white geometric outline, on a dark green background with black branches.</t>
+          <t>A pale ribbed surreal figure in profile with a hammer in its head and a red anatomical heart outside the body inside a white geometric outline, on a dark green background with black branches.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3855,10 +4095,15 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
+          <t>A pale, thin figure with a visible spine stands in profile with a hammer stuck in its head, while a red heart sits outside its body inside a white outline. This is surrealism: impossible, dreamlike images used to show feelings. The hammer may stand for pain, pressure or a thought that hurts, and the separated heart for emotions cut off from the body. Dark green and bare black branches make the mood heavy and unsettling.</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
           <t>Hammer and Heart</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="Q49" t="inlineStr">
         <is>
           <t>[{"hex": "#282926", "pct": 43.1}, {"hex": "#364934", "pct": 23.9}, {"hex": "#ccc1be", "pct": 15.9}, {"hex": "#ac9595", "pct": 6.8}, {"hex": "#81695c", "pct": 6.0}, {"hex": "#7b2933", "pct": 4.3}]</t>
         </is>
@@ -3892,7 +4137,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>A dark still life with a crystal wine glass, a dark vase holding a branch of tiny white flowers, and two golden-yellow fruits on a table. Small colorful flower dots and white sparkles are scattered over the dark background like confetti or stars. A signature is in the lower right.</t>
+          <t>A dark still life with a crystal wine glass, a dark vase holding a branch of tiny white flowers, and two golden-yellow fruits on a table. Small colorful flower dots and white sparkles are scattered over the dark background like confetti or stars.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3935,7 +4180,12 @@
           <t>objects in the lower left on a diagonal table edge, flowers rising upward</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>A crystal wine glass, a vase with tiny white flowers and two golden fruits sit on a table in a dark setting, with sparkles and small flower dots floating around them. The dark background makes the objects glow, a classic still-life trick. The scattered sparkles turn a quiet table into something magical, like stars or confetti. It may be read as a still life of a special evening or celebration.</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
         <is>
           <t>[{"hex": "#726a61", "pct": 23.5}, {"hex": "#8c8479", "pct": 22.1}, {"hex": "#504942", "pct": 18.1}, {"hex": "#2c2828", "pct": 15.6}, {"hex": "#aea593", "pct": 14.1}, {"hex": "#cfcbbd", "pct": 6.6}]</t>
         </is>
@@ -4012,7 +4262,12 @@
           <t>central rectangular image of angels inside a rough painted border</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Images of golden-haloed angels in a Renaissance style are set into a crumpled, painted surface in red, orange, green and gold. This is a collage: the artist reuses famous-looking religious images and places them in a new, rough setting. The contrast between the delicate angels and the crumpled texture can suggest how old sacred images live on in modern times. The singing angels give it a festive, heavenly mood.</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
         <is>
           <t>[{"hex": "#ab8067", "pct": 28.4}, {"hex": "#875a4b", "pct": 21.5}, {"hex": "#b6ab97", "pct": 17.6}, {"hex": "#828977", "pct": 12.9}, {"hex": "#436c5a", "pct": 9.8}, {"hex": "#3c3c38", "pct": 9.7}]</t>
         </is>
@@ -4089,7 +4344,12 @@
           <t>fish hanging vertically in two pairs on a central sheet</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr">
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Four fish hang on strings in front of a crumpled white sheet, two golden and two silver. Hanging fish are a traditional still-life subject, linked to food, markets and daily life. The crumpled background and fine lines make the picture about textures: scales, paper and light. It is a quiet, almost stark image that asks us to look closely at simple things.</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
         <is>
           <t>[{"hex": "#766d63", "pct": 20.9}, {"hex": "#5c544d", "pct": 20.7}, {"hex": "#90887d", "pct": 18.8}, {"hex": "#ada697", "pct": 17.4}, {"hex": "#cbc5b8", "pct": 11.3}, {"hex": "#3f3a35", "pct": 10.9}]</t>
         </is>
@@ -4123,7 +4383,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>A ballerina in a dramatic forward bend, with her dark hair in a bun and her legs extended in a bent pose. She is painted in white and grey against dark blue-grey vertical drips. A signature 'Bacho' appears in the lower right.</t>
+          <t>A ballerina in a dramatic forward bend, with her dark hair in a bun and her legs extended in a bent pose. She is painted in white and grey against dark blue-grey vertical drips.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -4166,7 +4426,12 @@
           <t>figure filling the vertical frame on a diagonal</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>A ballerina bends deeply forward, her body and legs forming a strong curved shape. She is painted in white and grey against dark vertical drips, so she seems to glow out of the darkness. Ballet looks effortless but takes great strength, and this pose shows both grace and tension. The dark background may add a feeling of loneliness or of a dancer alone on stage.</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
         <is>
           <t>[{"hex": "#c4bcb2", "pct": 23.9}, {"hex": "#a8a39d", "pct": 21.2}, {"hex": "#838583", "pct": 15.4}, {"hex": "#d7d1ca", "pct": 15.0}, {"hex": "#596265", "pct": 13.4}, {"hex": "#373d42", "pct": 11.1}]</t>
         </is>
@@ -4200,7 +4465,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>A loose, washed cityscape with grey-blue building facades on the right and pink and brown horizontal bands suggesting rooftops and sky. Grey clouds sit in a pale sky. White columns and dripping strokes are visible, with a signature in the lower right.</t>
+          <t>A loose, washed cityscape with grey-blue building facades on the right and pink and brown horizontal bands suggesting rooftops and sky. Grey clouds sit in a pale sky. White columns and dripping strokes are visible.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4243,7 +4508,12 @@
           <t>building mass on the right, horizontal bands on the left</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr">
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>A city at dusk is suggested by washes of grey-blue buildings and pink and brown bands of sky and rooftops. The paint drips and blends, so the scene looks wet and soft, like seeing the city through rain or tired eyes. Instead of details, the artist captures light and atmosphere. It may be read as the quiet moment when the day ends and the city fades into evening.</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
         <is>
           <t>[{"hex": "#646259", "pct": 22.6}, {"hex": "#928c86", "pct": 19.8}, {"hex": "#c5c3bc", "pct": 18.0}, {"hex": "#817064", "pct": 17.9}, {"hex": "#aba7a0", "pct": 12.1}, {"hex": "#4d5047", "pct": 9.6}]</t>
         </is>
@@ -4307,10 +4577,15 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
+          <t>An old town scene: a stone bridge with lamp posts, a tall evergreen tree and an old house with a wooden balcony by the river. Wooden balconies like these are typical of historic neighborhoods in many old cities. The warm light and loose brushwork make the place feel lived-in and familiar. It may be read as an affectionate portrait of an old part of town.</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
           <t>Old Bridge</t>
         </is>
       </c>
-      <c r="P55" t="inlineStr">
+      <c r="Q55" t="inlineStr">
         <is>
           <t>[{"hex": "#a3a5a0", "pct": 22.9}, {"hex": "#b7bab7", "pct": 18.0}, {"hex": "#796e5f", "pct": 16.9}, {"hex": "#8c8882", "pct": 16.9}, {"hex": "#5d5544", "pct": 15.0}, {"hex": "#3e3730", "pct": 10.4}]</t>
         </is>
@@ -4339,7 +4614,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>A long horizontal drawing of a hilly landscape with scattered houses, small trees, a few pink blossoming trees and grazing animals. Blue mountains run along the top. It is drawn with charcoal and colored crayon on cream paper and signed in the lower right.</t>
+          <t>A long horizontal drawing of a hilly landscape with scattered houses, small trees, a few pink blossoming trees and grazing animals. Blue mountains run along the top. It is drawn with charcoal and colored crayon on cream paper.</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4382,7 +4657,12 @@
           <t>wide panoramic band, mountains at the top edge</t>
         </is>
       </c>
-      <c r="P56" t="inlineStr">
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>A long, wide drawing shows rolling hills with small houses, trees, a few blossoming trees and grazing animals, with blue mountains along the top. The panoramic format makes us scan the land from left to right like a journey. It is drawn quickly with charcoal and crayon, more like an artist's sketch from nature. It gives a calm, spacious feeling of countryside and village life.</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
         <is>
           <t>[{"hex": "#8d8779", "pct": 28.1}, {"hex": "#777265", "pct": 22.0}, {"hex": "#a49e95", "pct": 18.1}, {"hex": "#b3b3b3", "pct": 13.6}, {"hex": "#56554f", "pct": 12.3}, {"hex": "#2b2d2c", "pct": 6.0}]</t>
         </is>
@@ -4401,7 +4681,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>A soft pastel landscape of rounded hills in ochre, pink, grey and violet patches. A single red tree with a black trunk stands in the lower right. A signature is in the lower right corner.</t>
+          <t>A soft pastel landscape of rounded hills in ochre, pink, grey and violet patches. A single red tree with a black trunk stands in the lower right.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4446,10 +4726,15 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
+          <t>Soft, rounded hills in ochre, pink, grey and violet fill the picture, with a single red tree in the corner. Pastel colors blend gently, so the landscape feels warm and dreamy. The lone red tree stands out as the only strong accent, catching your eye. It may be read as a symbol of individuality or simply a bright moment in a quiet landscape.</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
           <t>Red Tree</t>
         </is>
       </c>
-      <c r="P57" t="inlineStr">
+      <c r="Q57" t="inlineStr">
         <is>
           <t>[{"hex": "#9b908e", "pct": 28.2}, {"hex": "#7d7878", "pct": 21.8}, {"hex": "#715c56", "pct": 16.7}, {"hex": "#9a775b", "pct": 15.6}, {"hex": "#adb0b3", "pct": 12.5}, {"hex": "#572730", "pct": 5.1}]</t>
         </is>
@@ -4468,7 +4753,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>A simple pastel landscape with three green trees with black trunks on an ochre ground. Behind them are blue hills, and a single black bird flies in a pale grey sky. A signature is in the lower right.</t>
+          <t>A simple pastel landscape with three green trees with black trunks on an ochre ground. Behind them are blue hills, and a single black bird flies in a pale grey sky.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -4513,10 +4798,15 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
+          <t>Three green trees stand on ochre ground in front of blue hills, while a single black bird flies across a pale sky. The scene is drawn in a very simple, almost childlike way, which makes it calm and honest. The small bird adds a sense of life and freedom to the still landscape. It is a peaceful picture of the countryside.</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
           <t>Three Trees</t>
         </is>
       </c>
-      <c r="P58" t="inlineStr">
+      <c r="Q58" t="inlineStr">
         <is>
           <t>[{"hex": "#939895", "pct": 28.0}, {"hex": "#b1b1ad", "pct": 21.6}, {"hex": "#34689b", "pct": 17.7}, {"hex": "#9b724e", "pct": 14.9}, {"hex": "#43605d", "pct": 13.5}, {"hex": "#262425", "pct": 4.3}]</t>
         </is>
@@ -4535,7 +4825,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>A vase of flowers on a brown background: red poppies with black centers and white daisies with yellow centers above a dark, squat black vase. Green leaves are dabbed between the flowers. A signature is in the lower right.</t>
+          <t>A vase of flowers on a brown background: red poppies with black centers and white daisies with yellow centers above a dark, squat black vase. Green leaves are dabbed between the flowers.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -4580,10 +4870,15 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
+          <t>Red poppies and white daisies stand in a dark, low vase against a brown background. The flowers are painted with quick, simple dabs, giving the picture a fresh, spontaneous feel. Red and white against brown make the bouquet pop out from the dark. Flowers in a vase are a classic subject that celebrates simple everyday beauty.</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
           <t>Poppies and Daisies</t>
         </is>
       </c>
-      <c r="P59" t="inlineStr">
+      <c r="Q59" t="inlineStr">
         <is>
           <t>[{"hex": "#6e655c", "pct": 31.4}, {"hex": "#8b7b6a", "pct": 24.9}, {"hex": "#4a4a4c", "pct": 19.0}, {"hex": "#a89a85", "pct": 10.1}, {"hex": "#c2736b", "pct": 7.6}, {"hex": "#cdd0ce", "pct": 7.0}]</t>
         </is>
@@ -4602,7 +4897,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>A landscape with a pale ochre hill and a stone tower or fortress on top, with dark blue and pink shapes suggesting trees or buildings. Strong reflections of the photographer and the room on the glass obscure most of the lower half.</t>
+          <t>A landscape with a pale ochre hill and a stone tower or fortress on top, with dark blue and pink shapes suggesting trees or buildings.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4637,7 +4932,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>obscured by glass reflections</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4647,10 +4942,15 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
+          <t>A stone tower or fortress stands on top of a pale hill, surrounded by dark shapes like trees or buildings. Hilltop towers often appear in landscapes as symbols of history and protection. The tower is the clear focus. It may be read as a peaceful view of an old landmark.</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
           <t>Fortress on the Hill</t>
         </is>
       </c>
-      <c r="P60" t="inlineStr">
+      <c r="Q60" t="inlineStr">
         <is>
           <t>[{"hex": "#a59c8c", "pct": 23.1}, {"hex": "#b7b7b4", "pct": 21.6}, {"hex": "#6c6451", "pct": 21.6}, {"hex": "#87755c", "pct": 13.1}, {"hex": "#858584", "pct": 11.0}, {"hex": "#4e4940", "pct": 9.5}]</t>
         </is>
@@ -4727,7 +5027,12 @@
           <t>building dominating the right, tree on the left, small figures at the bottom</t>
         </is>
       </c>
-      <c r="P61" t="inlineStr">
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>A tall building with a red awning and orange flowers rises over a sidewalk café where small figures sit and walk. The thick paint and bright light give it a sunny, cheerful feel. Street cafés like this are a symbol of city life and relaxing outdoors. The small people make the building look grand and the street lively.</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
         <is>
           <t>[{"hex": "#aba8aa", "pct": 32.8}, {"hex": "#81888f", "pct": 23.9}, {"hex": "#514a30", "pct": 15.8}, {"hex": "#3a5a82", "pct": 10.7}, {"hex": "#241822", "pct": 9.7}, {"hex": "#a54146", "pct": 7.0}]</t>
         </is>
@@ -4804,7 +5109,12 @@
           <t>central rectangle surrounded by broad strokes</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr">
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Broad strokes of grey-green, olive, ochre and terracotta form a loose space with a frame-like rectangle in the middle, maybe a window or doorway. The scene is painted so freely that it sits between a real room and an abstract painting. The earthy colors give it a calm, muted mood. It invites you to imagine what is beyond the rectangle.</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
         <is>
           <t>[{"hex": "#676861", "pct": 24.7}, {"hex": "#827f79", "pct": 20.7}, {"hex": "#a19e92", "pct": 16.9}, {"hex": "#775042", "pct": 16.6}, {"hex": "#c2c3c1", "pct": 12.1}, {"hex": "#423a37", "pct": 9.1}]</t>
         </is>
@@ -4881,7 +5191,12 @@
           <t>two figures facing each other across a central table</t>
         </is>
       </c>
-      <c r="P63" t="inlineStr">
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Two young men in ancient-looking tunics sit on stools playing backgammon, one holding a dice cup, in front of a row of columns. Backgammon is one of the oldest board games in the world and is still very popular in many countries. Placing a modern-looking game in an ancient setting creates a playful mix of past and present. It may be read as a joke about how little some human habits change over time.</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
         <is>
           <t>[{"hex": "#879092", "pct": 37.0}, {"hex": "#a5afb0", "pct": 30.4}, {"hex": "#834031", "pct": 13.4}, {"hex": "#332922", "pct": 6.7}, {"hex": "#355c66", "pct": 6.4}, {"hex": "#b97629", "pct": 6.1}]</t>
         </is>
@@ -4958,7 +5273,12 @@
           <t>building mass on the left, portico right, chandelier upper center</t>
         </is>
       </c>
-      <c r="P64" t="inlineStr">
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>A large dark building with a tower and columns stands under a pale sky, while a chandelier floats in mid-air in front of it. An indoor object outside, hanging from nowhere, is a surreal idea that makes us look twice. The heavy, dark building and the strange light stripes create a mysterious, dreamlike mood. It may be read as a memory of a grand place, where inside and outside mix together.</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
         <is>
           <t>[{"hex": "#bbc5bc", "pct": 23.2}, {"hex": "#8c7f82", "pct": 19.6}, {"hex": "#716468", "pct": 18.8}, {"hex": "#5a4c51", "pct": 14.3}, {"hex": "#b2ab90", "pct": 13.8}, {"hex": "#403237", "pct": 10.4}]</t>
         </is>
@@ -5030,7 +5350,12 @@
           <t>dark rectangular block in the center against vertical grey strokes</t>
         </is>
       </c>
-      <c r="P65" t="inlineStr">
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>A dark, faded image of figures in historical costume appears inside a field of scraped grey and white strokes, as if an old photograph or engraving is disappearing. Using worn, half-erased images is a way to talk about memory and the past fading away. The figures seem to belong to an elegant, aristocratic world that is now gone. The mood is melancholic and ghostly.</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
         <is>
           <t>[{"hex": "#a29e96", "pct": 25.5}, {"hex": "#b2afa7", "pct": 20.8}, {"hex": "#8f8b82", "pct": 19.2}, {"hex": "#4d4a48", "pct": 13.5}, {"hex": "#c5c4be", "pct": 12.1}, {"hex": "#736f69", "pct": 8.9}]</t>
         </is>
@@ -5094,10 +5419,15 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
+          <t>Thousands of tiny blue leaf-like marks are arranged in sweeping curved rows over a warm orange-red ground. The rows bend like wind through grass or waves on water. This kind of patient, repeated mark-making creates rhythm and makes the surface feel alive. It may be read as a celebration of nature's patterns and movement.</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
           <t>Autumn Wind</t>
         </is>
       </c>
-      <c r="P66" t="inlineStr">
+      <c r="Q66" t="inlineStr">
         <is>
           <t>[{"hex": "#a37834", "pct": 21.1}, {"hex": "#ac826f", "pct": 19.2}, {"hex": "#b54322", "pct": 18.7}, {"hex": "#64757c", "pct": 15.1}, {"hex": "#614a3c", "pct": 13.5}, {"hex": "#94a1af", "pct": 12.3}]</t>
         </is>
@@ -5161,10 +5491,15 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
+          <t>Green leaves, each with a small orange streak, cover the whole canvas, with tiny colored dots between them. There is no single focal point, so your eye wanders across the surface as if looking into a bush or garden. Repeating one motif many times creates a calming, rhythmic pattern. It may be read as an image of growth and the richness of plant life.</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
           <t>Green Leaves</t>
         </is>
       </c>
-      <c r="P67" t="inlineStr">
+      <c r="Q67" t="inlineStr">
         <is>
           <t>[{"hex": "#209668", "pct": 30.2}, {"hex": "#198340", "pct": 29.6}, {"hex": "#4ba77a", "pct": 16.1}, {"hex": "#2690aa", "pct": 10.7}, {"hex": "#917c37", "pct": 8.3}, {"hex": "#83b5b9", "pct": 5.0}]</t>
         </is>
@@ -5183,7 +5518,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Pale pink four-petaled blossoms with yellow centers drift across a deep blue-violet background with pink and turquoise bands near the top. Thin white curved lines trail behind the flowers like wind. A signature beginning 'Gel...' appears on the right edge.</t>
+          <t>Pale pink four-petaled blossoms with yellow centers drift across a deep blue-violet background with pink and turquoise bands near the top. Thin white curved lines trail behind the flowers like wind.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -5228,10 +5563,15 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
+          <t>Pale pink blossoms drift across a deep blue-violet sky, with thin white lines trailing behind them like wind. The dark background makes the flowers look like they are glowing or floating at night. Falling blossoms are often a symbol of spring and of beauty that does not last long. The picture has a soft, dreamy mood.</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
           <t>Spring Blossoms</t>
         </is>
       </c>
-      <c r="P68" t="inlineStr">
+      <c r="Q68" t="inlineStr">
         <is>
           <t>[{"hex": "#323798", "pct": 37.8}, {"hex": "#5f4c93", "pct": 15.6}, {"hex": "#dfc4ce", "pct": 15.1}, {"hex": "#6985a9", "pct": 12.3}, {"hex": "#cc98a5", "pct": 11.7}, {"hex": "#a35f7c", "pct": 7.6}]</t>
         </is>
@@ -5250,7 +5590,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>A night scene of many small white birds with red breasts perched on thin white lines like wires or branches against a black textured sky. A larger white bird flies near the top beside a small moon, and a large pale bird shape rests near the bottom center. The image is framed by a violet-blue painted border; the photo is slightly blurred.</t>
+          <t>A night scene of many small white birds with red breasts perched on thin white lines like wires or branches against a black textured sky. A larger white bird flies near the top beside a small moon, and a large pale bird shape rests near the bottom center. The image is framed by a violet-blue painted border.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -5295,10 +5635,15 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
+          <t>Many small white birds with red breasts sit on thin lines like wires or branches against a black night sky, with a small moon above. The repetition of the birds creates a rhythm, almost like musical notes on a staff. The dark background and white birds suggest a cold winter night. It may be read as a quiet, slightly mysterious image of nature resting.</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
           <t>Winter Birds</t>
         </is>
       </c>
-      <c r="P69" t="inlineStr">
+      <c r="Q69" t="inlineStr">
         <is>
           <t>[{"hex": "#3d4247", "pct": 37.9}, {"hex": "#545a61", "pct": 19.4}, {"hex": "#777a83", "pct": 12.6}, {"hex": "#7284b9", "pct": 11.9}, {"hex": "#a4a3ab", "pct": 9.6}, {"hex": "#d2d1d5", "pct": 8.6}]</t>
         </is>
@@ -5317,7 +5662,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>An all-over pattern of gold leaf-like shapes with fine orange veins, small dark dots and short turquoise brushstrokes on a reddish ground. The shapes swirl in many directions. Part of a gold frame is visible on the right.</t>
+          <t>An all-over pattern of gold leaf-like shapes with fine orange veins, small dark dots and short turquoise brushstrokes on a reddish ground. The shapes swirl in many directions.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -5362,10 +5707,15 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
+          <t>Golden leaf shapes with fine orange veins swirl across a red ground, with small dark dots and touches of turquoise. The metallic gold gives the painting a rich, decorative shine. The swirling direction of the leaves suggests wind or movement. It may be read as an image of autumn, warmth or abundance.</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
           <t>Golden Leaves</t>
         </is>
       </c>
-      <c r="P70" t="inlineStr">
+      <c r="Q70" t="inlineStr">
         <is>
           <t>[{"hex": "#885542", "pct": 31.9}, {"hex": "#a27f71", "pct": 22.9}, {"hex": "#58342d", "pct": 17.9}, {"hex": "#c3b9aa", "pct": 13.9}, {"hex": "#4d607a", "pct": 8.6}, {"hex": "#61a6c9", "pct": 4.8}]</t>
         </is>
@@ -5384,7 +5734,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>A dense abstract field of diagonal streaks in red, pink, green and purple, covered with small pink and turquoise dots. The strokes radiate as if from a burst. The photo is slightly blurred and has a light reflection on the right.</t>
+          <t>A dense abstract field of diagonal streaks in red, pink, green and purple, covered with small pink and turquoise dots. The strokes radiate as if from a burst.</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -5419,7 +5769,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>no depicted light source; glare on right</t>
+          <t>no depicted light source</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5427,7 +5777,12 @@
           <t>all-over diagonal radiating strokes</t>
         </is>
       </c>
-      <c r="P71" t="inlineStr">
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Diagonal streaks of red, pink, green and purple radiate across the canvas, scattered with small dots. The lines spread as if from an explosion or a burst of light. Strong colors and dense marks create a lot of energy. It may be read as fireworks, a flower opening or simply a burst of joy.</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
         <is>
           <t>[{"hex": "#3a3b3b", "pct": 24.0}, {"hex": "#918d96", "pct": 19.7}, {"hex": "#62676d", "pct": 17.1}, {"hex": "#6d434a", "pct": 15.1}, {"hex": "#9a646f", "pct": 12.3}, {"hex": "#c2a3af", "pct": 11.9}]</t>
         </is>
@@ -5491,10 +5846,15 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
+          <t>Rows of small house-like shapes with violet roofs and bare blue trees fill a burgundy and pink field, while white dots fall like snow. The repeated houses make the village feel like a pattern or a textile. The lighter right side suggests distant light or fog. It may be read as a quiet winter village seen in a dream or memory.</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
           <t>Winter Village</t>
         </is>
       </c>
-      <c r="P72" t="inlineStr">
+      <c r="Q72" t="inlineStr">
         <is>
           <t>[{"hex": "#74374c", "pct": 20.9}, {"hex": "#a794bc", "pct": 18.4}, {"hex": "#987297", "pct": 17.9}, {"hex": "#572331", "pct": 17.2}, {"hex": "#885170", "pct": 16.3}, {"hex": "#c1b2e0", "pct": 9.3}]</t>
         </is>
@@ -5556,7 +5916,12 @@
           <t>all-over repeating rounded forms</t>
         </is>
       </c>
-      <c r="P73" t="inlineStr">
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Rounded pink and mauve shapes outlined in turquoise cover the canvas like cells, pebbles or petals. Patterns that look like living cells remind us of nature seen under a microscope. The repetition and soft colors make the surface calm but intricate. It may be read as an image of growth, life or the hidden patterns inside things.</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
         <is>
           <t>[{"hex": "#928c99", "pct": 21.1}, {"hex": "#514851", "pct": 18.5}, {"hex": "#34262a", "pct": 16.6}, {"hex": "#ababb9", "pct": 16.2}, {"hex": "#885d6e", "pct": 14.7}, {"hex": "#5c7884", "pct": 13.0}]</t>
         </is>
@@ -5620,10 +5985,15 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
+          <t>A plant with spiky turquoise and red leaves bursts upward from the bottom center, in front of yellow lines that suggest windows or furniture. The scene looks like a house plant in a bright room, simplified into patterns. The upward burst gives the picture energy, like a fountain. It may be read as a celebration of life growing indoors.</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
           <t>Green Interior</t>
         </is>
       </c>
-      <c r="P74" t="inlineStr">
+      <c r="Q74" t="inlineStr">
         <is>
           <t>[{"hex": "#30603b", "pct": 21.4}, {"hex": "#757062", "pct": 20.6}, {"hex": "#448850", "pct": 19.9}, {"hex": "#619490", "pct": 16.7}, {"hex": "#92b6b3", "pct": 11.2}, {"hex": "#b6b742", "pct": 10.1}]</t>
         </is>
@@ -5687,10 +6057,15 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
+          <t>Thin reddish branches spread across a pale blue-grey ground covered with tiny dots and squiggles like blossoms. The branches come from one corner, which creates a strong diagonal movement across the picture. The fine, patient detail feels delicate and airy. It may be read as a branch in spring bloom.</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
           <t>Blossoming Branch</t>
         </is>
       </c>
-      <c r="P75" t="inlineStr">
+      <c r="Q75" t="inlineStr">
         <is>
           <t>[{"hex": "#979b97", "pct": 26.5}, {"hex": "#a9afac", "pct": 24.4}, {"hex": "#8d8175", "pct": 16.0}, {"hex": "#c2c7c3", "pct": 12.9}, {"hex": "#76878f", "pct": 11.1}, {"hex": "#67655b", "pct": 9.2}]</t>
         </is>
@@ -5754,10 +6129,15 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
+          <t>Small light-blue flowers, brown round shapes and green leaves cover the whole surface, linked by thin golden swirls. The evenly filled surface turns a meadow into a decorative pattern, a bit like embroidery or a carpet. The tiny blue flowers resemble forget-me-nots, often a symbol of memory and love. It is a cheerful, detailed piece that rewards close looking.</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
           <t>Forget-me-nots</t>
         </is>
       </c>
-      <c r="P76" t="inlineStr">
+      <c r="Q76" t="inlineStr">
         <is>
           <t>[{"hex": "#5b5f5a", "pct": 28.4}, {"hex": "#484745", "pct": 26.4}, {"hex": "#767677", "pct": 18.6}, {"hex": "#979695", "pct": 12.2}, {"hex": "#70bdcc", "pct": 7.6}, {"hex": "#b4c7c2", "pct": 6.9}]</t>
         </is>
@@ -5791,7 +6171,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>An abstract of pinkish-violet hatched diagonal stripes forming zigzag bands, with wavy blue and red lines at the top. Small round yellow and green circles with dark centers, like eyes or seeds, are scattered across. A signature is in the lower right and part of a gold frame shows at the bottom.</t>
+          <t>An abstract of pinkish-violet hatched diagonal stripes forming zigzag bands, with wavy blue and red lines at the top. Small round yellow and green circles with dark centers, like eyes or seeds, are scattered across.</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -5834,7 +6214,12 @@
           <t>horizontal bands at top, diagonal hatching below</t>
         </is>
       </c>
-      <c r="P77" t="inlineStr">
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>Pinkish-violet stripes form zigzag bands, with wavy blue and red lines at the top and small round circles like eyes or seeds scattered across. The repeated diagonals create a strong rhythm, almost like music or woven fabric. The circles add a sense of something watching or growing. It is an abstract design about pattern and rhythm.</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
         <is>
           <t>[{"hex": "#998da5", "pct": 28.6}, {"hex": "#b5a1b2", "pct": 23.0}, {"hex": "#86738a", "pct": 20.7}, {"hex": "#aa8183", "pct": 10.4}, {"hex": "#cec3d0", "pct": 8.8}, {"hex": "#655d73", "pct": 8.5}]</t>
         </is>
@@ -5911,7 +6296,12 @@
           <t>light central mass framed by dark edges</t>
         </is>
       </c>
-      <c r="P78" t="inlineStr">
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>A light center of white, cream and ochre is surrounded by deep teal, navy, mustard and maroon. Putting the lightest colors in the middle makes the center glow, as if light is breaking through. The paint is layered and scraped, which gives it a rough, earthy texture. Like many abstract works, it is about color and feeling rather than a specific subject.</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
         <is>
           <t>[{"hex": "#5c584d", "pct": 23.1}, {"hex": "#383c38", "pct": 20.0}, {"hex": "#976f4f", "pct": 16.1}, {"hex": "#7a7874", "pct": 15.2}, {"hex": "#a9967f", "pct": 15.0}, {"hex": "#bbb2a9", "pct": 10.6}]</t>
         </is>
@@ -5940,7 +6330,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>An abstract painting dominated by warm pink, rust and peach shapes resembling two rounded forms or figures, outlined by dark teal arcs. A glare of light reflects in the upper center. The background edges are muted brown.</t>
+          <t>An abstract painting dominated by warm pink, rust and peach shapes resembling two rounded forms or figures, outlined by dark teal arcs. The background edges are muted brown.</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -5975,7 +6365,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>glare on surface, no depicted source</t>
+          <t>no depicted light source</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5983,7 +6373,12 @@
           <t>two rounded masses side by side, dark arcs between them</t>
         </is>
       </c>
-      <c r="P79" t="inlineStr">
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>Warm pink, rust and peach shapes form two rounded masses, separated by dark teal curves. The rounded forms can look like two figures or bodies leaning together, though nothing is clearly drawn. Warm colors give the painting an intimate, gentle mood. It may be read as an image of closeness, but the artist leaves it open.</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
         <is>
           <t>[{"hex": "#895c52", "pct": 30.7}, {"hex": "#58524b", "pct": 21.3}, {"hex": "#a68074", "pct": 17.9}, {"hex": "#777773", "pct": 15.2}, {"hex": "#b4aaa2", "pct": 9.1}, {"hex": "#e3e6de", "pct": 5.7}]</t>
         </is>
@@ -6047,7 +6442,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>no depicted light source; glare on surface</t>
+          <t>no depicted light source</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6055,7 +6450,12 @@
           <t>warm left half versus cool blue right</t>
         </is>
       </c>
-      <c r="P80" t="inlineStr">
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>Bright yellow, fiery red and orange crowd the left side, while a deep blue patch sits on the right. The contrast between hot and cold colors creates tension, like fire meeting sky or water. Energetic brushwork makes the whole surface feel alive. It may be read as an emotional or natural force, but there is no single correct interpretation.</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
         <is>
           <t>[{"hex": "#5e5b5d", "pct": 21.1}, {"hex": "#261b17", "pct": 20.4}, {"hex": "#a38136", "pct": 17.9}, {"hex": "#74381b", "pct": 15.9}, {"hex": "#989490", "pct": 15.4}, {"hex": "#e4ddda", "pct": 9.4}]</t>
         </is>
@@ -6119,7 +6519,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>no depicted light source; glare on surface</t>
+          <t>no depicted light source</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -6127,7 +6527,12 @@
           <t>light left side, dark right side</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr">
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Soft violet and lavender on the left meet dark charcoal and teal masses on the right, with small red and orange sparks in between. The painting moves from light to dark across its width, like a change of mood or weather. The thick, glossy paint makes the surface rich and physical. It invites you to feel the shift from calm to heavy.</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
         <is>
           <t>[{"hex": "#696662", "pct": 25.7}, {"hex": "#b09d93", "pct": 21.7}, {"hex": "#8c817c", "pct": 20.4}, {"hex": "#4a4743", "pct": 16.2}, {"hex": "#b57144", "pct": 8.2}, {"hex": "#d4c5b9", "pct": 7.8}]</t>
         </is>
@@ -6199,7 +6604,12 @@
           <t>dark central vertical mass with lighter edges</t>
         </is>
       </c>
-      <c r="P82" t="inlineStr">
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>Broad, layered strokes of dusty pink, ochre, rust and slate blue fill a tall canvas, with a dark blue-black column running down the middle. The dark central band acts like a spine that holds the composition together. The blended, thick paint gives it a soft but heavy feel. It is an abstract work about color and mood, and viewers may read the dark center as something serious or hidden.</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
         <is>
           <t>[{"hex": "#b09d8c", "pct": 21.6}, {"hex": "#544a48", "pct": 17.8}, {"hex": "#cdbda7", "pct": 15.7}, {"hex": "#9b7866", "pct": 15.6}, {"hex": "#6b6d6e", "pct": 14.7}, {"hex": "#8a8c91", "pct": 14.6}]</t>
         </is>
@@ -6263,7 +6673,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>no depicted light source; glare in the center</t>
+          <t>no depicted light source</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -6271,7 +6681,12 @@
           <t>warm mass at the top, cooler darker base</t>
         </is>
       </c>
-      <c r="P83" t="inlineStr">
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>A fiery mass of red, orange and yellow fills the upper half, resting on darker greys, mauves and blues below. Warm colors on top and cool, dark ones underneath create a feeling of fire rising or energy bursting upward. A tiny bright blue spot near the center gives the eye a place to rest. It may be read as passion, heat or a sunset, though it shows no specific subject.</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
         <is>
           <t>[{"hex": "#686566", "pct": 30.3}, {"hex": "#91817a", "pct": 27.2}, {"hex": "#4a3c3f", "pct": 13.3}, {"hex": "#bbb087", "pct": 10.8}, {"hex": "#9e3e34", "pct": 10.5}, {"hex": "#d5921f", "pct": 7.9}]</t>
         </is>
@@ -6335,7 +6750,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>no depicted light source; glare on surface</t>
+          <t>no depicted light source</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -6343,7 +6758,12 @@
           <t>dark central field with yellow fragments scattered around it</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr">
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>Jagged shards of bright orange-yellow break through a dark charcoal field. The sharp, angular shapes feel like cracks of light or sparks in darkness. The strong contrast between dark and bright makes the painting dramatic and tense. It may be read as hope or light breaking through difficult times.</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
         <is>
           <t>[{"hex": "#3d3d3c", "pct": 35.0}, {"hex": "#656266", "pct": 24.9}, {"hex": "#898888", "pct": 16.9}, {"hex": "#7f5932", "pct": 10.0}, {"hex": "#de9516", "pct": 8.4}, {"hex": "#b3bec8", "pct": 4.8}]</t>
         </is>
@@ -6420,7 +6840,12 @@
           <t>two figures centered, crossing stems, cat bottom right</t>
         </is>
       </c>
-      <c r="P85" t="inlineStr">
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>Two women in long white dresses stand side by side, each holding a tall stem with large teal leaves, and an orange cat sits at their feet. One has lighter skin and auburn hair, the other darker skin and dark hair, and their matching dresses and poses suggest equality and friendship. The warm orange and pink background makes the scene peaceful and sunny. It may be read as a picture of togetherness across differences.</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
         <is>
           <t>[{"hex": "#afb1aa", "pct": 31.5}, {"hex": "#a67762", "pct": 19.9}, {"hex": "#985d38", "pct": 18.9}, {"hex": "#573020", "pct": 12.0}, {"hex": "#83afba", "pct": 9.9}, {"hex": "#1f627a", "pct": 7.7}]</t>
         </is>
@@ -6492,7 +6917,12 @@
           <t>sofa across the center, dragonflies above and below</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr">
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>In a soft green garden, a woman with a red flower instead of a head sits on a flowery sofa while another woman sleeps with her head in her lap. Giant dragonflies float around them. Replacing a head with a flower is a surreal idea, often used to show dreams or inner feelings. The calm colors and the sleeping figure suggest a spring daydream where nature and people blend.</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
         <is>
           <t>[{"hex": "#9c928d", "pct": 28.3}, {"hex": "#867f76", "pct": 20.7}, {"hex": "#6f6c60", "pct": 15.9}, {"hex": "#b0a5a3", "pct": 13.9}, {"hex": "#555648", "pct": 12.9}, {"hex": "#34362a", "pct": 8.3}]</t>
         </is>
@@ -6569,7 +6999,12 @@
           <t>groups on left and right, deer and stream in the center, cliffs behind</t>
         </is>
       </c>
-      <c r="P87" t="inlineStr">
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>A dramatic scene in a dark forest: a crowd in historical dress gathers around a kneeling man, a half-naked figure stands near the rocks, and a small deer lies by a stream in the center. The deer and the stream form the quiet focus between the two groups, as if something important has just happened there. Dark varnished colors and a stormy sky give the scene the feel of an old legend or historical event, perhaps about a hunt and a discovery.</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
         <is>
           <t>[{"hex": "#353a3b", "pct": 21.3}, {"hex": "#938c83", "pct": 17.8}, {"hex": "#535653", "pct": 17.0}, {"hex": "#72706b", "pct": 15.4}, {"hex": "#212123", "pct": 15.3}, {"hex": "#b3a69b", "pct": 13.3}]</t>
         </is>
@@ -6646,7 +7081,12 @@
           <t>seated figure centered and filling the vertical frame</t>
         </is>
       </c>
-      <c r="P88" t="inlineStr">
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>An old man with a long beard, fur hat and long coat sits holding a cane, with a dagger at his belt. Fierce black brushstrokes and scratches surround him and partly dissolve his figure, as if he is emerging from memory or from the mountains themselves. His clothing suggests a traditional mountain culture. The portrait feels serious and dignified, honoring a wise elder or important figure.</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
         <is>
           <t>[{"hex": "#191815", "pct": 21.5}, {"hex": "#c3bab3", "pct": 21.0}, {"hex": "#a39b94", "pct": 15.5}, {"hex": "#393530", "pct": 15.4}, {"hex": "#807872", "pct": 13.6}, {"hex": "#5d5750", "pct": 13.0}]</t>
         </is>
@@ -6710,10 +7150,15 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
+          <t>Large sweeping arcs of orange, red and green circle across a light turquoise ground, with small splashes of yellow and blue. The curved lines create a strong feeling of spinning or swirling motion. Bright, warm colors on a cool background make the movement pop. It may be read as wind, dance or pure energy.</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
           <t>Orange Whirl</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr">
+      <c r="Q89" t="inlineStr">
         <is>
           <t>[{"hex": "#d86e46", "pct": 29.2}, {"hex": "#9f573d", "pct": 21.0}, {"hex": "#99c1c3", "pct": 18.5}, {"hex": "#b68d79", "pct": 11.0}, {"hex": "#505246", "pct": 10.5}, {"hex": "#669693", "pct": 9.9}]</t>
         </is>
@@ -6790,7 +7235,12 @@
           <t>centered frontal half-figure, buckets around the edges</t>
         </is>
       </c>
-      <c r="P90" t="inlineStr">
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>A woman with long wavy hair and a checkered jacket looks straight at us, holding a long red paintbrush, while red paint buckets float in a blue sky around her. The direct gaze and the brush suggest that she is an artist presenting herself. Floating buckets in the sky is a surreal touch, as if her imagination is spilling into the world. It may be read as a confident self-portrait about creativity.</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
         <is>
           <t>[{"hex": "#b2b0a5", "pct": 29.1}, {"hex": "#03366e", "pct": 18.5}, {"hex": "#1c1918", "pct": 15.1}, {"hex": "#07558c", "pct": 14.0}, {"hex": "#673633", "pct": 12.3}, {"hex": "#9c7b69", "pct": 11.0}]</t>
         </is>
@@ -6867,7 +7317,12 @@
           <t>figure filling the frame, dandelions upper left</t>
         </is>
       </c>
-      <c r="P91" t="inlineStr">
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>A girl wrapped in a large teal cloak with tiny flowers holds a bunch of white dandelion clocks, tilting her face toward them. Blowing on dandelions to make a wish is a childhood tradition in many places. The warm, scratched background and simple shapes give it a gentle, storybook feel. It may be read as an image of childhood, wishes and innocence.</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
         <is>
           <t>[{"hex": "#4b6a73", "pct": 19.6}, {"hex": "#bd9e7f", "pct": 19.4}, {"hex": "#2b4751", "pct": 18.1}, {"hex": "#7b888b", "pct": 17.7}, {"hex": "#d7c1aa", "pct": 15.9}, {"hex": "#825b3e", "pct": 9.3}]</t>
         </is>
@@ -6944,7 +7399,12 @@
           <t>all-over foliage with denser area in the center</t>
         </is>
       </c>
-      <c r="P92" t="inlineStr">
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>Pale leaf and branch silhouettes are layered over a deep cobalt blue background, like shadows of plants on a wall. The leaves look printed or stenciled, a technique that captures the exact shapes of real plants. Faint chair legs at the bottom hint at a room. It may be read as a quiet interior where plants and their shadows create a living pattern.</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
         <is>
           <t>[{"hex": "#baa88c", "pct": 25.1}, {"hex": "#95937e", "pct": 20.5}, {"hex": "#d0bfa5", "pct": 15.2}, {"hex": "#315a80", "pct": 15.0}, {"hex": "#697873", "pct": 14.7}, {"hex": "#4379a5", "pct": 9.4}]</t>
         </is>
@@ -7021,7 +7481,12 @@
           <t>diagonal chair shape crossing the frame, plant in the center</t>
         </is>
       </c>
-      <c r="P93" t="inlineStr">
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>Translucent shapes of a chair and leafy stems overlap on a dark blue and teal background, with a bright green grid in the corner. The misty, layered effect looks like a print or a double exposure in photography. Everyday objects become ghostly silhouettes. It may be read as a memory of a room or a garden, where objects and plants blend together.</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
         <is>
           <t>[{"hex": "#8f936f", "pct": 23.1}, {"hex": "#636a50", "pct": 20.8}, {"hex": "#a5b092", "pct": 19.4}, {"hex": "#324856", "pct": 17.0}, {"hex": "#55867c", "pct": 10.7}, {"hex": "#c9cab2", "pct": 9.1}]</t>
         </is>
@@ -7040,7 +7505,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>A doll-like child figure with a pale face, large golden wig and gold puffed costume rides a rearing white horse with a red saddle and bridle against a dark green background. A golden feathered hat floats above the head, and golden clouds drift in the sky. Initials 'O.T.' appear in the lower right.</t>
+          <t>A doll-like child figure with a pale face, large golden wig and gold puffed costume rides a rearing white horse with a red saddle and bridle against a dark green background. A golden feathered hat floats above the head, and golden clouds drift in the sky.</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -7085,10 +7550,15 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
+          <t>A doll-like child with a huge golden wig and puffed gold costume rides a rearing white horse, with a feathered hat floating above. This plays with old royal portraits, where kings were shown proudly on horseback to show power. Turning the ruler into a small doll-like child makes the grand tradition funny and ironic. It may be read as gentle humor about power, vanity and childhood.</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
           <t>Little Prince on a White Horse</t>
         </is>
       </c>
-      <c r="P94" t="inlineStr">
+      <c r="Q94" t="inlineStr">
         <is>
           <t>[{"hex": "#1a361b", "pct": 47.6}, {"hex": "#43522f", "pct": 15.3}, {"hex": "#8c702d", "pct": 14.1}, {"hex": "#beb8a7", "pct": 12.0}, {"hex": "#a89464", "pct": 7.7}, {"hex": "#a62c20", "pct": 3.3}]</t>
         </is>
@@ -7107,7 +7577,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>A doll-like child figure with a pale face and big golden wig, in a gold puffed costume, rides a white horse with golden harness against a bright red background. A golden feathered hat floats above and golden clouds drift around. Initials 'O.T.' appear in the lower right.</t>
+          <t>A doll-like child figure with a pale face and big golden wig, in a gold puffed costume, rides a white horse with golden harness against a bright red background. A golden feathered hat floats above and golden clouds drift around.</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -7152,10 +7622,15 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
+          <t>A doll-like child in a golden wig and gold costume rides a white horse against a bright red background, with a feathered hat floating above. It plays with the tradition of royal portraits on horseback, which were meant to show strength and power. The toy-like figure and floating hat make it playful and ironic instead of serious. The flat red background makes the golden figure stand out like an icon.</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
           <t>Little Prince on a Red Ground</t>
         </is>
       </c>
-      <c r="P95" t="inlineStr">
+      <c r="Q95" t="inlineStr">
         <is>
           <t>[{"hex": "#a31626", "pct": 25.8}, {"hex": "#b7324b", "pct": 20.4}, {"hex": "#957153", "pct": 19.4}, {"hex": "#bdc6c7", "pct": 14.3}, {"hex": "#ab9d80", "pct": 13.5}, {"hex": "#543d31", "pct": 6.6}]</t>
         </is>
@@ -7219,10 +7694,15 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
+          <t>A doll-like girl in a dark green court gown with gold trim and puffed sleeves stands stiffly with her arms out, a green feathered hat floating above her head. Her look recalls old royal portraits of young princesses in huge formal dresses. The stiff pose and floating hat make it humorous, as if she is a toy dressed up for an official portrait. It may be read as a playful comment on royalty and the weight of tradition on children.</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
           <t>Infanta in Green</t>
         </is>
       </c>
-      <c r="P96" t="inlineStr">
+      <c r="Q96" t="inlineStr">
         <is>
           <t>[{"hex": "#2f3b33", "pct": 55.7}, {"hex": "#2a2925", "pct": 20.3}, {"hex": "#5e5236", "pct": 7.9}, {"hex": "#95743d", "pct": 7.4}, {"hex": "#d1c7bc", "pct": 5.0}, {"hex": "#b19c64", "pct": 3.8}]</t>
         </is>
@@ -7299,7 +7779,12 @@
           <t>symmetrical centered standing figure</t>
         </is>
       </c>
-      <c r="P97" t="inlineStr">
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>A doll-like girl in a crimson court gown with gold stripes stands stiffly with outstretched arms, a red feathered hat floating above her. The pose and costume recall formal royal portraits of young princesses. The black background and flat style make her look like a toy on display. It may be read as gentle irony about royal pomp and how children were treated as symbols.</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
         <is>
           <t>[{"hex": "#7e2738", "pct": 36.2}, {"hex": "#2e2b28", "pct": 34.6}, {"hex": "#5e3c33", "pct": 12.4}, {"hex": "#87674e", "pct": 9.3}, {"hex": "#ad9475", "pct": 5.3}, {"hex": "#d5cdc9", "pct": 2.2}]</t>
         </is>
@@ -7376,7 +7861,12 @@
           <t>radiating burst left of center over all-over splatter</t>
         </is>
       </c>
-      <c r="P98" t="inlineStr">
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Fine white lines and splashes radiate across a black and grey ground, crossed by thin threads of red, turquoise, orange and pink. The paint was dripped and flung, a technique where the artist's movement becomes the image. The radiating lines suggest an explosion or a burst of light. It may be read as chaos, energy or a night full of sparks.</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
         <is>
           <t>[{"hex": "#6d6a68", "pct": 20.8}, {"hex": "#4c4a4a", "pct": 19.1}, {"hex": "#8d8986", "pct": 18.9}, {"hex": "#b0aba5", "pct": 15.9}, {"hex": "#272729", "pct": 14.0}, {"hex": "#d4d0ca", "pct": 11.3}]</t>
         </is>
@@ -7453,7 +7943,12 @@
           <t>tall central figure with the child in the lower center</t>
         </is>
       </c>
-      <c r="P99" t="inlineStr">
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>A tall, elongated woman in green holds a yellow round object like a balloon, while a small red-haired girl stands in front of her. The stretched figure and soft violet background give the scene a dreamy, magical feel. The closeness of the two figures suggests a mother and child or a protector. It may be read as a tender image of care, dreams and childhood.</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
         <is>
           <t>[{"hex": "#9d998e", "pct": 30.4}, {"hex": "#808081", "pct": 28.9}, {"hex": "#8a8b51", "pct": 13.5}, {"hex": "#586e42", "pct": 11.6}, {"hex": "#c3a750", "pct": 8.8}, {"hex": "#d9cda0", "pct": 6.9}]</t>
         </is>
@@ -7487,7 +7982,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>A woman with a stylized pale face, one large blue eye and a hand raised to her lips, wears a richly colored dress made of thick multicolored dabs. A small green hat sits on her head and the background is muted grey-green. A signature appears in the lower right.</t>
+          <t>A woman with a stylized pale face, one large blue eye and a hand raised to her lips, wears a richly colored dress made of thick multicolored dabs. A small green hat sits on her head and the background is muted grey-green.</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -7530,7 +8025,12 @@
           <t>half-figure filling the vertical frame</t>
         </is>
       </c>
-      <c r="P100" t="inlineStr">
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>A woman with a stylized pale face, one large eye and a hand to her lips wears a dress built from thick dabs of many colors. Her face is simplified, almost like a mask, while her dress is rich and busy, a playful contrast. The hand at her lips suggests thought, shyness or a secret. It can be read as a portrait of an elegant, thoughtful lady.</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
         <is>
           <t>[{"hex": "#988f82", "pct": 27.0}, {"hex": "#7f796c", "pct": 25.3}, {"hex": "#605c55", "pct": 14.9}, {"hex": "#c7b09d", "pct": 12.6}, {"hex": "#363438", "pct": 11.6}, {"hex": "#d7ccc4", "pct": 8.5}]</t>
         </is>
@@ -7607,7 +8107,12 @@
           <t>shed upper left, tree right, cow and children in the foreground</t>
         </is>
       </c>
-      <c r="P101" t="inlineStr">
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>A village scene: a wooden shed, a woman feeding geese, a fruit tree, a white cow and two children in the front. A real weathered wooden plank is attached to the bottom, bringing an actual piece of village life into the painting. The muted colors and simple figures give it a nostalgic, storytelling mood. It may be read as a memory of childhood in the countryside.</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
         <is>
           <t>[{"hex": "#98957c", "pct": 24.9}, {"hex": "#827f66", "pct": 24.5}, {"hex": "#69684f", "pct": 17.2}, {"hex": "#b0ac98", "pct": 16.2}, {"hex": "#474936", "pct": 11.1}, {"hex": "#d4d5d0", "pct": 6.1}]</t>
         </is>
@@ -7679,7 +8184,12 @@
           <t>old building in the lower half, new city stacked behind, vertical format</t>
         </is>
       </c>
-      <c r="P102" t="inlineStr">
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>An old red-brown building with balconies and hanging laundry stands in front of modern white high-rises and construction cranes. The painting puts old and new side by side, showing a city that is changing fast. The old house feels personal and lived-in, while the new towers feel cold and unfinished. It may be read as a reflection on what is lost and gained when cities modernize.</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
         <is>
           <t>[{"hex": "#6a4d3d", "pct": 22.2}, {"hex": "#708988", "pct": 21.8}, {"hex": "#9e9f90", "pct": 17.5}, {"hex": "#84725d", "pct": 17.4}, {"hex": "#3c3129", "pct": 14.3}, {"hex": "#c4c3b8", "pct": 6.9}]</t>
         </is>
@@ -7756,7 +8266,12 @@
           <t>elephant in profile filling the horizontal frame</t>
         </is>
       </c>
-      <c r="P103" t="inlineStr">
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>A large elephant with long tusks walks across the canvas, built from small triangles and squares like a mosaic, with a golden sun-like circle behind it. Breaking a subject into geometric pieces is a cubist idea that lets the artist play with shape and color. The zebra-like stripes inside its body mix different animals in one image. It may be read as a celebration of wild animals and their strength.</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
         <is>
           <t>[{"hex": "#62665e", "pct": 20.5}, {"hex": "#413d39", "pct": 19.6}, {"hex": "#859692", "pct": 19.0}, {"hex": "#9c744c", "pct": 14.2}, {"hex": "#bdbaa0", "pct": 13.9}, {"hex": "#bd9f62", "pct": 12.9}]</t>
         </is>
@@ -7828,7 +8343,12 @@
           <t>figures across the upper half on a diagonal, village at bottom center</t>
         </is>
       </c>
-      <c r="P104" t="inlineStr">
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>Three long-haired women in flowing dresses float through a shimmering sky, two of them blowing long trumpets, with stars, a crescent moon and a tiny row of houses below. Floating figures and trumpets often stand for celebration, announcement or heavenly music. The horizontal, glittering strokes make the sky feel alive and magical. It may be read as a festive dream over a sleeping town.</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
         <is>
           <t>[{"hex": "#906d4e", "pct": 24.6}, {"hex": "#a28d6f", "pct": 21.7}, {"hex": "#7b4739", "pct": 21.0}, {"hex": "#6a6e6a", "pct": 12.8}, {"hex": "#4c3f43", "pct": 10.9}, {"hex": "#aeac9e", "pct": 9.0}]</t>
         </is>
@@ -7900,7 +8420,12 @@
           <t>figures interlocked across the center</t>
         </is>
       </c>
-      <c r="P105" t="inlineStr">
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>Two figures are intertwined in an embrace, one pale and nude, the other in yellow and white, surrounded by crusty turquoise, violet and rust paint. The thick, rough texture makes the figures feel like they are emerging from the paint itself. The embrace suggests love, closeness or passion. It may be read as an intense image of intimacy.</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
         <is>
           <t>[{"hex": "#37312f", "pct": 20.0}, {"hex": "#4b5c5e", "pct": 17.2}, {"hex": "#708487", "pct": 16.6}, {"hex": "#826243", "pct": 16.3}, {"hex": "#ae8f62", "pct": 16.2}, {"hex": "#c2beac", "pct": 13.7}]</t>
         </is>
@@ -7972,7 +8497,12 @@
           <t>torso filling the vertical frame, head top left</t>
         </is>
       </c>
-      <c r="P106" t="inlineStr">
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>A nude female torso, seen from behind and in profile, glows in warm ochre, rust and gold against a dark blue background. The nude is one of the oldest subjects in art, used to study the body, light and beauty. Thick scraped paint gives the skin warmth and texture. It may be read as a calm, sensual study of the human form.</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
         <is>
           <t>[{"hex": "#633d2d", "pct": 24.0}, {"hex": "#86613c", "pct": 20.6}, {"hex": "#2a2c36", "pct": 18.6}, {"hex": "#9a845e", "pct": 17.6}, {"hex": "#535e68", "pct": 13.0}, {"hex": "#bdb38e", "pct": 6.3}]</t>
         </is>
@@ -8036,10 +8566,15 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
+          <t>A white hillside town with blue-domed churches and stacked cube-shaped houses looks out over the sea. This style of architecture is famous on some Mediterranean islands, where white walls reflect the strong sun. The image is so realistic that it is close to a photograph. It celebrates light, sea and a peaceful island atmosphere.</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
           <t>Blue Domes</t>
         </is>
       </c>
-      <c r="P107" t="inlineStr">
+      <c r="Q107" t="inlineStr">
         <is>
           <t>[{"hex": "#98928a", "pct": 32.8}, {"hex": "#bbb09e", "pct": 20.2}, {"hex": "#d3cdbd", "pct": 15.4}, {"hex": "#373136", "pct": 13.2}, {"hex": "#7d634e", "pct": 12.8}, {"hex": "#667fa6", "pct": 5.6}]</t>
         </is>
@@ -8103,10 +8638,15 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
+          <t>Three children with big heads and sleepy, half-closed eyes stand in a row; two hold paper boats and the middle one holds an egg-like object on a strange machine. Paper boats are a classic symbol of childhood play and imagination. Their tired, serious faces add a touch of melancholy to a playful scene. It may be read as a picture of childhood dreams mixed with a hint of sadness.</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
           <t>Paper Boats</t>
         </is>
       </c>
-      <c r="P108" t="inlineStr">
+      <c r="Q108" t="inlineStr">
         <is>
           <t>[{"hex": "#88382a", "pct": 20.2}, {"hex": "#2d7689", "pct": 19.9}, {"hex": "#3f463e", "pct": 17.0}, {"hex": "#907a5a", "pct": 16.7}, {"hex": "#c4a840", "pct": 14.8}, {"hex": "#c4ccbd", "pct": 11.4}]</t>
         </is>
@@ -8170,10 +8710,15 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
+          <t>A tropical village of colorful stilt houses with corrugated roofs crowds the waterside, with palm leaves and laundry between them. Stilt houses are built to stay above water and floods in many tropical regions. The bright colors and energetic strokes make the scene feel busy and full of life. It may be read as a lively portrait of everyday life by the water.</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
           <t>Houses on Stilts</t>
         </is>
       </c>
-      <c r="P109" t="inlineStr">
+      <c r="Q109" t="inlineStr">
         <is>
           <t>[{"hex": "#5c6655", "pct": 24.3}, {"hex": "#937a54", "pct": 17.3}, {"hex": "#373934", "pct": 16.7}, {"hex": "#84938f", "pct": 16.4}, {"hex": "#b9c0b8", "pct": 13.2}, {"hex": "#bfaa7b", "pct": 12.0}]</t>
         </is>
@@ -8192,7 +8737,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>A tall thin standing figure wrapped in a red cloak, with a dark head, large round earrings and a long staff, stands on a white background. Splatters and drips of red and yellow ochre paint cover the background. A signature is at the bottom.</t>
+          <t>A tall thin standing figure wrapped in a red cloak, with a dark head, large round earrings and a long staff, stands on a white background. Splatters and drips of red and yellow ochre paint cover the background.</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -8237,10 +8782,15 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
+          <t>A tall, thin figure wrapped in a red cloak, with large round earrings and a long staff, stands alone on a white background splattered with red and ochre paint. The red cloak, earrings and staff resemble the traditional dress of Maasai warriors in East Africa. The splatters add energy around the still figure. It may be read as a proud, dignified portrait of a warrior.</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
           <t>Maasai Warrior</t>
         </is>
       </c>
-      <c r="P110" t="inlineStr">
+      <c r="Q110" t="inlineStr">
         <is>
           <t>[{"hex": "#bbb19c", "pct": 32.1}, {"hex": "#c9c5b3", "pct": 29.4}, {"hex": "#ad9a7f", "pct": 20.9}, {"hex": "#9c7451", "pct": 8.5}, {"hex": "#732e2a", "pct": 5.6}, {"hex": "#271413", "pct": 3.6}]</t>
         </is>
@@ -8304,10 +8854,15 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
+          <t>A huge crowd of small figures in bright clothes gathers below a hillside of houses with corrugated roofs. The crowd is painted with quick vertical dabs, so it feels busy and moving. Such scenes often show markets, festivals or community gatherings. It may be read as a celebration of community and lively village life.</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
           <t>Market Day</t>
         </is>
       </c>
-      <c r="P111" t="inlineStr">
+      <c r="Q111" t="inlineStr">
         <is>
           <t>[{"hex": "#8f6c50", "pct": 21.4}, {"hex": "#4f4840", "pct": 18.6}, {"hex": "#a09e8e", "pct": 17.9}, {"hex": "#637a77", "pct": 15.1}, {"hex": "#c9cbbc", "pct": 14.8}, {"hex": "#bea456", "pct": 12.2}]</t>
         </is>
@@ -8371,10 +8926,15 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
+          <t>Five tall women in red, blue and black wraps stand together, wearing large beaded collars and earrings, one carrying sticks on her head and another a gourd. Beaded collars like these are part of traditional dress in some East African communities. Standing close together, the women look strong and united. It may be read as a proud portrait of women, tradition and daily work.</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
           <t>Five Women</t>
         </is>
       </c>
-      <c r="P112" t="inlineStr">
+      <c r="Q112" t="inlineStr">
         <is>
           <t>[{"hex": "#cdcdc3", "pct": 38.8}, {"hex": "#393030", "pct": 14.0}, {"hex": "#a03d3b", "pct": 14.0}, {"hex": "#a68d85", "pct": 13.7}, {"hex": "#695f57", "pct": 11.2}, {"hex": "#355b90", "pct": 8.3}]</t>
         </is>
@@ -8438,10 +8998,15 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
+          <t>Three slender women with raised arms and grass skirts dance across a textured gold and green background, overlaid with circles and lines like a star map. The repeated poses create a rhythm, like a ritual dance. The cosmic shapes may connect the dance to nature, the sky or spiritual beliefs. The sandy texture makes the surface feel ancient and earthy.</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
           <t>Three Dancers</t>
         </is>
       </c>
-      <c r="P113" t="inlineStr">
+      <c r="Q113" t="inlineStr">
         <is>
           <t>[{"hex": "#81957b", "pct": 21.7}, {"hex": "#627361", "pct": 20.8}, {"hex": "#ab9f76", "pct": 20.6}, {"hex": "#91835f", "pct": 16.0}, {"hex": "#b8bd95", "pct": 10.7}, {"hex": "#404644", "pct": 10.3}]</t>
         </is>
@@ -8503,7 +9068,12 @@
           <t>all-over vertical strokes</t>
         </is>
       </c>
-      <c r="P114" t="inlineStr">
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Thick palette-knife strokes of yellow, white, blue, green and red crowd the canvas. The marks look like a crowd of people or flags moving in the wind, though nothing is clearly drawn. Using a palette knife leaves bold, sculpted paint. It may be read as a festival or crowd seen in a blur of color.</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
         <is>
           <t>[{"hex": "#5e684e", "pct": 21.5}, {"hex": "#879070", "pct": 18.5}, {"hex": "#2e4746", "pct": 17.3}, {"hex": "#957137", "pct": 15.2}, {"hex": "#b3bca3", "pct": 13.9}, {"hex": "#c0a832", "pct": 13.6}]</t>
         </is>
@@ -8522,7 +9092,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>A rural Southeast Asian scene with thatched houses on stilts, laundry hanging on a line, and tall trees and mountains under a grey sky. A woman carries two baskets on a shoulder pole across a pale dirt road. 'NOY 2015' and 'Vientiane, Laos' are written in the lower left.</t>
+          <t>A rural Southeast Asian scene with thatched houses on stilts, laundry hanging on a line, and tall trees and mountains under a grey sky. A woman carries two baskets on a shoulder pole across a pale dirt road. 'Vientiane, Laos' is written in the lower left.</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -8567,10 +9137,15 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
+          <t>A Southeast Asian village of thatched houses on stilts sits beneath tall trees and misty mountains, while a woman carries two baskets on a shoulder pole. The writing on the painting names Vientiane, Laos. The grey sky and soft colors give it a calm, everyday mood. It is a respectful portrait of rural life and work.</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
           <t>Village near Vientiane</t>
         </is>
       </c>
-      <c r="P115" t="inlineStr">
+      <c r="Q115" t="inlineStr">
         <is>
           <t>[{"hex": "#bcb7ae", "pct": 23.9}, {"hex": "#a79e8e", "pct": 20.1}, {"hex": "#89806a", "pct": 16.9}, {"hex": "#d5d2cb", "pct": 14.7}, {"hex": "#645d49", "pct": 13.0}, {"hex": "#36352b", "pct": 11.5}]</t>
         </is>
@@ -8634,10 +9209,15 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
+          <t>A narrow old street leads toward an ornate gate with an arch, past a church tower and decorated buildings. The perspective of the street pulls your eye straight to the gate. Thick paint and soft light give the scene a nostalgic, old-world atmosphere. It may be read as an invitation to walk through a historic European town.</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
           <t>Street to the Gate</t>
         </is>
       </c>
-      <c r="P116" t="inlineStr">
+      <c r="Q116" t="inlineStr">
         <is>
           <t>[{"hex": "#c8c9c6", "pct": 26.8}, {"hex": "#7c7563", "pct": 18.6}, {"hex": "#989180", "pct": 17.2}, {"hex": "#b4afa1", "pct": 15.5}, {"hex": "#5d5345", "pct": 13.5}, {"hex": "#352f2a", "pct": 8.4}]</t>
         </is>
@@ -8701,10 +9281,15 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
+          <t>A woman in a red jacket walks away from us under a white umbrella on a rainy street. The red jacket is the only bright color, so it instantly catches the eye in the grey scene. Thick palette-knife strokes make the rain and reflections feel wet and shimmering. It may be read as a quiet, solitary moment in the city.</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
           <t>Red Umbrella Walk</t>
         </is>
       </c>
-      <c r="P117" t="inlineStr">
+      <c r="Q117" t="inlineStr">
         <is>
           <t>[{"hex": "#aaab9d", "pct": 23.4}, {"hex": "#8e8d7e", "pct": 21.1}, {"hex": "#d1d1c5", "pct": 19.1}, {"hex": "#6e6b57", "pct": 15.7}, {"hex": "#463931", "pct": 14.5}, {"hex": "#a12f2e", "pct": 6.1}]</t>
         </is>
@@ -8768,10 +9353,15 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
+          <t>A crowd of women with black faces and arms, wearing white dresses and hats, gathers at a market with baskets and round fruits. The painting uses almost only black, white and cream, which makes it elegant and graphic. The repeated shapes create a rhythm, like a pattern. It may be read as a celebration of women's work and community at the market.</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
           <t>Market Women in White</t>
         </is>
       </c>
-      <c r="P118" t="inlineStr">
+      <c r="Q118" t="inlineStr">
         <is>
           <t>[{"hex": "#cec8c0", "pct": 40.4}, {"hex": "#beb4aa", "pct": 30.0}, {"hex": "#a79a8f", "pct": 11.7}, {"hex": "#1b1716", "pct": 8.1}, {"hex": "#82746b", "pct": 6.1}, {"hex": "#4e4541", "pct": 3.8}]</t>
         </is>
@@ -8835,10 +9425,15 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
+          <t>Women with black faces and arms, dressed in white with hats, gather at a market with baskets and round fruits. The limited black, white and cream palette makes the image stylish and graphic. One woman lifts a bunch of fruit, adding movement. It may be read as a lively, rhythmic picture of market life.</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
           <t>Market Women in White</t>
         </is>
       </c>
-      <c r="P119" t="inlineStr">
+      <c r="Q119" t="inlineStr">
         <is>
           <t>[{"hex": "#cfcac1", "pct": 30.3}, {"hex": "#c0b7ad", "pct": 29.9}, {"hex": "#ad9f94", "pct": 17.2}, {"hex": "#1f1b1b", "pct": 11.9}, {"hex": "#8a7b70", "pct": 7.2}, {"hex": "#524947", "pct": 3.5}]</t>
         </is>
@@ -8857,7 +9452,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>A black-and-white African village scene with thatched round huts on both sides of a path leading to the shore. Two palm trees rise in the center and a boat with a sail and two people floats on the water. Birds fly in the sky and a few figures stand by the huts; a signature is in the lower left.</t>
+          <t>A black-and-white African village scene with thatched round huts on both sides of a path leading to the shore. Two palm trees rise in the center and a boat with a sail and two people floats on the water. Birds fly in the sky and a few figures stand by the huts.</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -8902,10 +9497,15 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
+          <t>A village of thatched round huts lines a path leading to the shore, where a sailboat with two people floats between two palm trees. The black-and-white style makes the scene feel like a memory or an old photograph. The path leads your eye straight to the water and the boat. It may be read as a peaceful picture of coastal village life.</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
           <t>Village by the Sea</t>
         </is>
       </c>
-      <c r="P120" t="inlineStr">
+      <c r="Q120" t="inlineStr">
         <is>
           <t>[{"hex": "#272221", "pct": 23.9}, {"hex": "#d8d1ca", "pct": 19.5}, {"hex": "#4c4542", "pct": 16.0}, {"hex": "#b7afa8", "pct": 15.6}, {"hex": "#958d88", "pct": 14.2}, {"hex": "#716965", "pct": 10.9}]</t>
         </is>
@@ -8969,10 +9569,15 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
+          <t>Groups of tall women in red, blue and green wraps carry baskets and bundles on their heads under flat-topped acacia trees, with round huts nearby. Carrying loads on the head is a common daily practice in many rural African communities. The plain white background makes the colorful figures stand out like a frieze. It may be read as a portrait of daily village life and women's work.</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
           <t>Under the Acacias</t>
         </is>
       </c>
-      <c r="P121" t="inlineStr">
+      <c r="Q121" t="inlineStr">
         <is>
           <t>[{"hex": "#cecac1", "pct": 38.7}, {"hex": "#221f1d", "pct": 14.7}, {"hex": "#483d38", "pct": 13.5}, {"hex": "#b3aea6", "pct": 12.1}, {"hex": "#6a6159", "pct": 11.4}, {"hex": "#8d867f", "pct": 9.6}]</t>
         </is>
@@ -9036,10 +9641,15 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
+          <t>A floating village of thatched stilt houses sits on small islands in a calm lake, with people paddling narrow boats and temple towers on the far shore. Stilt houses and boats show a way of life closely tied to water. The pale, still water and soft colors make the scene peaceful and balanced, with the houses mirrored on both sides. It may be read as a calm, idealized view of life on the lake.</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
           <t>Floating Village</t>
         </is>
       </c>
-      <c r="P122" t="inlineStr">
+      <c r="Q122" t="inlineStr">
         <is>
           <t>[{"hex": "#d2cec7", "pct": 33.0}, {"hex": "#bdb8b2", "pct": 20.2}, {"hex": "#4c4544", "pct": 15.0}, {"hex": "#2c292c", "pct": 13.4}, {"hex": "#6e6966", "pct": 9.9}, {"hex": "#96908b", "pct": 8.5}]</t>
         </is>
@@ -9103,10 +9713,15 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
+          <t>Five women in white head wraps sit behind a market stall with baskets of red fruit, sliced watermelon and large golden clay pots. They are drawn with loose black outlines over gold, grey and white, which gives the image a sketch-like elegance. The row of women creates a rhythm across the top, while the goods fill the bottom. It may be read as a celebration of market life and women's work.</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
           <t>Watermelon Sellers</t>
         </is>
       </c>
-      <c r="P123" t="inlineStr">
+      <c r="Q123" t="inlineStr">
         <is>
           <t>[{"hex": "#968f85", "pct": 29.8}, {"hex": "#b6ad9c", "pct": 18.8}, {"hex": "#787167", "pct": 18.7}, {"hex": "#4c4236", "pct": 16.0}, {"hex": "#d6cfc3", "pct": 9.7}, {"hex": "#9c5e3d", "pct": 7.0}]</t>
         </is>
@@ -9183,7 +9798,12 @@
           <t>half-figure filling the vertical frame, face upper left</t>
         </is>
       </c>
-      <c r="P124" t="inlineStr">
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>A realistic portrait of a middle-aged man with greying hair, holding a microphone and a sheet of paper while touching his chin. The microphone and paper suggest he is giving a speech, reading or performing. His slight smile and thoughtful gesture make him seem warm and reflective. The blurred background keeps all attention on his face and hands.</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
         <is>
           <t>[{"hex": "#45392c", "pct": 24.9}, {"hex": "#221f1e", "pct": 19.5}, {"hex": "#2f3746", "pct": 17.0}, {"hex": "#58544f", "pct": 16.1}, {"hex": "#c19d75", "pct": 11.3}, {"hex": "#946f4a", "pct": 11.1}]</t>
         </is>
@@ -9255,7 +9875,12 @@
           <t>horizontal bands: sky top, hills middle, field bottom</t>
         </is>
       </c>
-      <c r="P125" t="inlineStr">
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>A blazing sunset fills the sky with orange and yellow above blue and purple hills, while the foreground glows red, green and turquoise. The paint is applied with a palette knife in thick ridges, so the colors almost burn on the surface. The colors are stronger than in real life, which turns the landscape into pure emotion. It may be read as the drama and warmth of the end of the day.</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
         <is>
           <t>[{"hex": "#c47f22", "pct": 22.4}, {"hex": "#263837", "pct": 20.6}, {"hex": "#a13a24", "pct": 18.1}, {"hex": "#406c7f", "pct": 15.5}, {"hex": "#896f5b", "pct": 12.6}, {"hex": "#a5a4a9", "pct": 10.8}]</t>
         </is>
@@ -9332,7 +9957,12 @@
           <t>figure upper left, desk diagonally in the lower right</t>
         </is>
       </c>
-      <c r="P126" t="inlineStr">
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>A man with swept-back hair sits at a large pale green desk or console, looking down at papers in a dim room. A soft spotlight glows at the top and faint figures appear in the background, as if he is on a stage or in a studio. The dark, theatrical lighting creates a focused, introspective mood. It may be read as a portrait of someone absorbed in his work or performance.</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
         <is>
           <t>[{"hex": "#413e3a", "pct": 25.4}, {"hex": "#575351", "pct": 24.3}, {"hex": "#2e231f", "pct": 22.2}, {"hex": "#746f63", "pct": 14.4}, {"hex": "#8f9084", "pct": 9.5}, {"hex": "#c8b6a6", "pct": 4.4}]</t>
         </is>
@@ -9409,7 +10039,12 @@
           <t>horizontal central band of images framed by patterned borders</t>
         </is>
       </c>
-      <c r="P127" t="inlineStr">
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>A strip of small naive-style pictures, a woman at a table, red houses with wooden balconies and figures in big hats, is set into crumpled fabric or paper printed with ferns. The central images look like a tribute to naive folk painting. Framing them with textured, patterned material makes the work feel like a scrapbook of memories. It may be read as an affectionate homage to old-town life and folk art.</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
         <is>
           <t>[{"hex": "#9b5e47", "pct": 26.5}, {"hex": "#7c3a2d", "pct": 21.3}, {"hex": "#a3846f", "pct": 18.2}, {"hex": "#353b34", "pct": 15.3}, {"hex": "#626254", "pct": 13.6}, {"hex": "#bcc1be", "pct": 5.1}]</t>
         </is>
@@ -9486,7 +10121,12 @@
           <t>high sky in the upper two thirds, landscape band below</t>
         </is>
       </c>
-      <c r="P128" t="inlineStr">
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>An evening landscape with a sky fading from blue to orange and pink, swirling purple clouds, a dark tree clump and a bridge in the distance. A red and white sign post on the right adds a modern touch. The loose brushwork and bright colors feel more like a feeling than an exact view. It may be read as a warm, dreamy memory of an evening by the river.</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
         <is>
           <t>[{"hex": "#a18f88", "pct": 25.6}, {"hex": "#63a5cd", "pct": 19.9}, {"hex": "#ce904d", "pct": 19.6}, {"hex": "#4e5d87", "pct": 14.0}, {"hex": "#534336", "pct": 11.9}, {"hex": "#c8cacd", "pct": 9.1}]</t>
         </is>
@@ -9563,7 +10203,12 @@
           <t>dark horizontal mass in the center surrounded by pale swirls</t>
         </is>
       </c>
-      <c r="P129" t="inlineStr">
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>Soft swirling cream, green and mauve shapes surround a dark burgundy and black mass cutting across the middle. The smooth blending and sharp dark silhouettes create a strange, almost cosmic scene. Small bright patches inside the dark area look like distant lights or planets. It may be read as an explosion, a galaxy or a powerful event in space.</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
         <is>
           <t>[{"hex": "#cdcebd", "pct": 27.8}, {"hex": "#b5b7a7", "pct": 22.6}, {"hex": "#21181d", "pct": 16.0}, {"hex": "#9f968b", "pct": 15.5}, {"hex": "#866f69", "pct": 9.3}, {"hex": "#5a3a3e", "pct": 8.8}]</t>
         </is>
@@ -9635,7 +10280,12 @@
           <t>overlapping blocks across the horizontal frame</t>
         </is>
       </c>
-      <c r="P130" t="inlineStr">
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>Broad blocks of peach, ochre, rust, brown and slate blue are outlined by dark lines, like overlapping planes or stacked shapes. The thick paint and visible strokes make the surface feel solid and physical. A small bright orange accent catches the eye in one corner. It is an abstract work about color, shape and balance, and invites you to find your own meaning.</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
         <is>
           <t>[{"hex": "#795236", "pct": 22.3}, {"hex": "#3c3e41", "pct": 21.3}, {"hex": "#b99770", "pct": 19.7}, {"hex": "#726d61", "pct": 14.3}, {"hex": "#c6bfae", "pct": 13.8}, {"hex": "#909893", "pct": 8.6}]</t>
         </is>
@@ -9669,7 +10319,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>A symmetrical mask-like face drawn in oil pastel with large oval eyes in rings of green, blue, pink and white, a long brown nose and an orange layered mouth. Purple, blue and orange shapes form the cheeks and ears. A border of short green and purple strokes surrounds the face; glare is visible on the glass.</t>
+          <t>A symmetrical mask-like face drawn in oil pastel with large oval eyes in rings of green, blue, pink and white, a long brown nose and an orange layered mouth. Purple, blue and orange shapes form the cheeks and ears. A border of short green and purple strokes surrounds the face.</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -9704,7 +10354,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>flat, with glare on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -9712,7 +10362,12 @@
           <t>symmetrical frontal face filling the frame</t>
         </is>
       </c>
-      <c r="P131" t="inlineStr">
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>A symmetrical, mask-like face is built from bright rings and shapes: big oval eyes, a long nose and a layered orange mouth, surrounded by a border of short colored strokes. Masks in many cultures are used in rituals, theater and celebrations to represent spirits or characters. The bold oil-pastel colors make it playful and powerful at the same time. It may be read as a joyful, folk-inspired face.</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
         <is>
           <t>[{"hex": "#bda194", "pct": 29.1}, {"hex": "#c5cac9", "pct": 17.0}, {"hex": "#ce7f36", "pct": 16.2}, {"hex": "#415152", "pct": 13.8}, {"hex": "#7e6373", "pct": 13.7}, {"hex": "#4b9093", "pct": 10.3}]</t>
         </is>
@@ -9746,7 +10401,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>A symmetrical abstract face built from bold bands: a red central nose shape flanked by blue and purple stripes, brown and pink eyebrow shapes, and a small red mouth near the bottom. Pale yellow, grey and light blue areas fill the background. Reflections of windows show on the glass.</t>
+          <t>A symmetrical abstract face built from bold bands: a red central nose shape flanked by blue and purple stripes, brown and pink eyebrow shapes, and a small red mouth near the bottom. Pale yellow, grey and light blue areas fill the background.</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -9781,7 +10436,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>flat, with reflections on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -9789,7 +10444,12 @@
           <t>vertical symmetry around the central red shape</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr">
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>A face is built from bold vertical bands: a red nose shape in the center, blue and purple stripes beside it, simple eyebrows and a small red mouth. Reducing a face to geometric shapes is a way to show its structure rather than its exact look. The symmetry gives it a mask-like, almost totem-like presence. It can be read as a playful experiment with how few shapes we need to recognize a face.</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
         <is>
           <t>[{"hex": "#c6b396", "pct": 20.8}, {"hex": "#d0ccbf", "pct": 19.2}, {"hex": "#91999a", "pct": 17.0}, {"hex": "#78666d", "pct": 14.8}, {"hex": "#cc3c3b", "pct": 14.4}, {"hex": "#38395b", "pct": 13.8}]</t>
         </is>
@@ -9866,7 +10526,12 @@
           <t>warm central mass with cooler right side</t>
         </is>
       </c>
-      <c r="P133" t="inlineStr">
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>Thick swirling strokes of red, coral, ochre and teal fill the canvas, with a dark curving line through the lower middle. The paint was applied wet into wet, so colors blend and move together. The curved black line gives the composition direction and tension. It is an abstract work about energy and color.</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
         <is>
           <t>[{"hex": "#985445", "pct": 22.8}, {"hex": "#6b7d7d", "pct": 19.4}, {"hex": "#b27d65", "pct": 17.1}, {"hex": "#ced3c5", "pct": 14.5}, {"hex": "#b4ab8c", "pct": 13.5}, {"hex": "#494d45", "pct": 12.7}]</t>
         </is>
@@ -9895,7 +10560,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>An abstract with two glowing yellow areas on the left and center, surrounded by dark maroon, grey and black strokes, with a bright blue stripe running down the middle. Ochre and orange appear at the right edge. The surface is glossy with a strong reflection at the bottom.</t>
+          <t>An abstract with two glowing yellow areas on the left and center, surrounded by dark maroon, grey and black strokes, with a bright blue stripe running down the middle. Ochre and orange appear at the right edge. The surface is glossy.</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -9930,7 +10595,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>no depicted light source; glare on surface</t>
+          <t>no depicted light source</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -9938,7 +10603,12 @@
           <t>two yellow focal points with dark surroundings</t>
         </is>
       </c>
-      <c r="P134" t="inlineStr">
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>Two glowing yellow areas shine out of dark maroon, grey and black strokes, with a bright blue stripe running down the middle. The bright colors stand out against the dark like lights in a night scene. The thick, glossy paint gives the surface depth. It may be read as light in darkness, or simply enjoyed as a strong contrast of colors.</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
         <is>
           <t>[{"hex": "#736e67", "pct": 32.1}, {"hex": "#90837b", "pct": 24.7}, {"hex": "#4f5f5f", "pct": 18.1}, {"hex": "#d0b46e", "pct": 14.0}, {"hex": "#9fa4a1", "pct": 7.8}, {"hex": "#e7dfcd", "pct": 3.2}]</t>
         </is>
@@ -10010,7 +10680,12 @@
           <t>warm masses around a cool central sweep</t>
         </is>
       </c>
-      <c r="P135" t="inlineStr">
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>Large patches of coral red, orange and ochre surround a vertical sweep of blue and purple, with a dark grey block in one corner and pale cream at the edges. The warm colors seem to push forward while the cool blue sinks back, creating depth. The gestural brushwork shows the artist's movement. It is an abstract composition about color, movement and feeling.</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
         <is>
           <t>[{"hex": "#6e7388", "pct": 21.6}, {"hex": "#c76b5d", "pct": 17.2}, {"hex": "#585e5b", "pct": 16.9}, {"hex": "#d2d5c7", "pct": 16.2}, {"hex": "#bf9989", "pct": 14.1}, {"hex": "#a5764b", "pct": 14.0}]</t>
         </is>
@@ -10087,7 +10762,12 @@
           <t>dense vertical mass filling the center</t>
         </is>
       </c>
-      <c r="P136" t="inlineStr">
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>Dense, streaky dark brown marks cover a pale surface, looking like fur, hair or tree bark. The marks were brushed or scraped mainly in one direction, which gives a strong sense of texture and growth. The work focuses on a single material quality rather than a picture. It may be read as an exploration of the body, hair or organic surfaces, making something ordinary look strange and fascinating.</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
         <is>
           <t>[{"hex": "#c9cdc1", "pct": 29.4}, {"hex": "#8b7569", "pct": 19.5}, {"hex": "#9f8e82", "pct": 17.1}, {"hex": "#765d52", "pct": 14.9}, {"hex": "#b4aea2", "pct": 12.6}, {"hex": "#5a3e35", "pct": 6.5}]</t>
         </is>
@@ -10164,7 +10844,12 @@
           <t>dense vertical mass with a curving left edge</t>
         </is>
       </c>
-      <c r="P137" t="inlineStr">
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>Dry, brushed dark brown streaks form a hairy, textured mass on a pale ground, with white gaps breaking through. It looks like fur or body hair seen very close. By focusing on texture alone, the work makes us think about the body and things we usually hide or ignore. It belongs together with a similar companion piece, like part of a series.</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
         <is>
           <t>[{"hex": "#c6c8bd", "pct": 21.3}, {"hex": "#7d6d63", "pct": 20.0}, {"hex": "#68554b", "pct": 18.5}, {"hex": "#92857a", "pct": 16.6}, {"hex": "#503931", "pct": 12.6}, {"hex": "#aaa298", "pct": 11.0}]</t>
         </is>
@@ -10236,7 +10921,12 @@
           <t>seated figure centered, filling the vertical frame</t>
         </is>
       </c>
-      <c r="P138" t="inlineStr">
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>A seated woman wears a hat topped with a blue fish and a slice of lemon, while her face is shown from the side and the front at the same time. Showing several viewpoints at once is a key idea of cubism. The fish hat is absurd and funny, turning a formal portrait into a playful one. It may be read as both a portrait and a joke about fashion and appearance.</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
         <is>
           <t>[{"hex": "#d3cbbd", "pct": 39.7}, {"hex": "#b6b5a6", "pct": 16.2}, {"hex": "#2d2d2e", "pct": 16.0}, {"hex": "#4584bb", "pct": 10.1}, {"hex": "#475a6f", "pct": 10.1}, {"hex": "#968974", "pct": 7.9}]</t>
         </is>
@@ -10255,7 +10945,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>A bold portrait of a bearded man with large dark eyes, a curling moustache and red lips, wearing a yellow and blue plumed hat and a red and white ruffled collar. The face is grey with heavy black brushstrokes. A date '5.6.4.69' and a signature are written at the top right.</t>
+          <t>A bold portrait of a bearded man with large dark eyes, a curling moustache and red lips, wearing a yellow and blue plumed hat and a red and white ruffled collar. The face is grey with heavy black brushstrokes.</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -10300,10 +10990,15 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
+          <t>A bold portrait of a bearded man with big dark eyes, a curling moustache, a plumed hat and a ruffled collar, painted with heavy black brushstrokes. His costume recalls 17th-century gentlemen or musketeers. The quick, confident strokes give him a lively, theatrical personality. It may be read as a playful character portrait inspired by old European paintings.</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
           <t>Musketeer</t>
         </is>
       </c>
-      <c r="P139" t="inlineStr">
+      <c r="Q139" t="inlineStr">
         <is>
           <t>[{"hex": "#a49e95", "pct": 38.3}, {"hex": "#c7c1b7", "pct": 17.9}, {"hex": "#69797a", "pct": 15.6}, {"hex": "#af252e", "pct": 11.4}, {"hex": "#3a3330", "pct": 11.3}, {"hex": "#d9a525", "pct": 5.5}]</t>
         </is>
@@ -10322,7 +11017,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>A portrait of a bearded man with a plumed purple hat, red hair or collar and one large eye, his face split into light and dark halves. His blue doublet has fern-like patterns with orange circles. The background is beige cardboard-like with a white patch on the right; a number and signature appear at the top and bottom.</t>
+          <t>A portrait of a bearded man with a plumed purple hat, red hair or collar and one large eye, his face split into light and dark halves. His blue doublet has fern-like patterns with orange circles. The background is beige cardboard-like with a white patch on the right.</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -10367,10 +11062,15 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
+          <t>A bearded man with a plumed hat and one large eye has his face split into light and dark halves, with a decorated blue doublet below. Splitting a face into contrasting parts is a way to show different sides of a person at once. The bright, flat colors and bold lines make him feel theatrical. It may be read as a playful, modern take on a historical character portrait.</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
           <t>Man with a Hat</t>
         </is>
       </c>
-      <c r="P140" t="inlineStr">
+      <c r="Q140" t="inlineStr">
         <is>
           <t>[{"hex": "#b8b19e", "pct": 32.0}, {"hex": "#a18a63", "pct": 29.2}, {"hex": "#637789", "pct": 14.5}, {"hex": "#2e3438", "pct": 11.3}, {"hex": "#a43a37", "pct": 8.4}, {"hex": "#d1861f", "pct": 4.7}]</t>
         </is>
@@ -10404,7 +11104,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>A white unicorn with a long flowing mane and a small flower on its horn stands on clouds. Thin leafy branches grow out of its back. The background is a sky-blue field sprinkled with gold specks and soft clouds; reflections on the glass are visible.</t>
+          <t>A white unicorn with a long flowing mane and a small flower on its horn stands on clouds. Thin leafy branches grow out of its back. The background is a sky-blue field sprinkled with gold specks and soft clouds.</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -10447,7 +11147,12 @@
           <t>unicorn in profile in the center of the horizontal frame</t>
         </is>
       </c>
-      <c r="P141" t="inlineStr">
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>A white unicorn with a flowing mane stands on clouds, with thin leafy branches growing out of its back and a small flower on its horn. Mixing animals with plants is a surrealist idea that creates impossible, dreamlike images. The soft blue sky with gold specks makes the scene magical. The unicorn, a symbol of purity and fantasy, becomes even more mysterious with nature growing from it.</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
         <is>
           <t>[{"hex": "#b5bcb7", "pct": 27.4}, {"hex": "#d0d0c4", "pct": 16.8}, {"hex": "#7a8189", "pct": 15.9}, {"hex": "#8fa1ac", "pct": 15.8}, {"hex": "#a79d90", "pct": 12.6}, {"hex": "#62676e", "pct": 11.5}]</t>
         </is>
@@ -10524,7 +11229,12 @@
           <t>arched format, sphere at the bottom, figures floating above</t>
         </is>
       </c>
-      <c r="P142" t="inlineStr">
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>An arched composition in deep blue looks like a stained-glass window, filled with floating animals, birds, a sun inside a sphere and Hebrew letters. Stained-glass windows often tell religious stories through symbols rather than realistic scenes. The animals and Hebrew text suggest biblical symbolism. The glowing colors and floating creatures give it a joyful, spiritual, dreamlike quality.</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
         <is>
           <t>[{"hex": "#5a6173", "pct": 27.5}, {"hex": "#81828c", "pct": 25.2}, {"hex": "#dad5be", "pct": 19.4}, {"hex": "#aca3a0", "pct": 15.0}, {"hex": "#44464a", "pct": 10.8}, {"hex": "#d0885f", "pct": 2.1}]</t>
         </is>
@@ -10601,7 +11311,12 @@
           <t>arched format, crown at top, lion in the lower half</t>
         </is>
       </c>
-      <c r="P143" t="inlineStr">
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>An arched, deep red composition resembling a stained-glass window shows two hands holding a crown above a roaring lion, with faint city walls and Hebrew text. The lion and the crown are traditional biblical symbols of kingship, often linked with the tribe of Judah. The bold red gives the image power and intensity. It may be read as a symbolic image of royalty, strength and faith.</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
         <is>
           <t>[{"hex": "#993939", "pct": 27.3}, {"hex": "#bf9692", "pct": 21.5}, {"hex": "#d0d0c6", "pct": 17.9}, {"hex": "#b36460", "pct": 16.0}, {"hex": "#57423f", "pct": 8.9}, {"hex": "#727176", "pct": 8.4}]</t>
         </is>
@@ -10635,7 +11350,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>A surreal flat composition with a grey airbrushed donkey standing on a pale green woven floor, its long braided tail curling up the left side. A dark bird flies at the top dropping pink blossoms, and grey stepped tower shapes and a colorful scale-patterned square stand behind. The background is white with a reflected window on the glass.</t>
+          <t>A surreal flat composition with a grey airbrushed donkey standing on a pale green woven floor, its long braided tail curling up the left side. A dark bird flies at the top dropping pink blossoms, and grey stepped tower shapes and a colorful scale-patterned square stand behind. The background is white.</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -10678,7 +11393,12 @@
           <t>donkey lower right, braid sweeping from left, bird top left</t>
         </is>
       </c>
-      <c r="P144" t="inlineStr">
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>A grey donkey with a long braided tail stands on a woven floor, while a dark bird drops pink blossoms from above, next to stepped towers and a colorful patterned square. The smooth airbrushed shapes and strange combinations create a surreal, puzzle-like scene. Nothing quite fits together logically, which invites us to make up our own story. It may be read as a dream or a playful mix of symbols.</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
         <is>
           <t>[{"hex": "#c1c1bd", "pct": 31.6}, {"hex": "#aaa79e", "pct": 30.6}, {"hex": "#676054", "pct": 13.7}, {"hex": "#86817a", "pct": 13.5}, {"hex": "#312c2b", "pct": 8.5}, {"hex": "#f7f8f9", "pct": 2.1}]</t>
         </is>
@@ -10755,7 +11475,12 @@
           <t>all-over writing across the horizontal frame</t>
         </is>
       </c>
-      <c r="P145" t="inlineStr">
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>Layers of chalky handwritten Georgian letters cover a grey wall-like surface, overlapping like graffiti or a used blackboard. The Georgian alphabet has its own unique, rounded script, and here the letters become shapes and rhythm rather than readable words. Writing over writing suggests memory, history and many voices. It may be read as a celebration of language and identity.</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
         <is>
           <t>[{"hex": "#95948f", "pct": 25.5}, {"hex": "#878380", "pct": 23.2}, {"hex": "#a6a69e", "pct": 20.3}, {"hex": "#b9b9ad", "pct": 14.6}, {"hex": "#746c6e", "pct": 9.8}, {"hex": "#cfd0c4", "pct": 6.6}]</t>
         </is>
@@ -10832,7 +11557,12 @@
           <t>vertical ochre form rising from a cluster at the bottom</t>
         </is>
       </c>
-      <c r="P146" t="inlineStr">
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>A large soft ochre shape with a dark cap rises from a cluster of cream and brown blobs, against a pale blue background. The forms look organic and melting, like living things or objects in a dream. Biomorphic shapes like these are inspired by nature and the body without copying them directly. The work is playful and strange, inviting you to imagine what the shapes might be.</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
         <is>
           <t>[{"hex": "#b3c0bd", "pct": 30.7}, {"hex": "#9baea9", "pct": 23.4}, {"hex": "#c8d1d2", "pct": 19.4}, {"hex": "#a37c3e", "pct": 10.3}, {"hex": "#c5a469", "pct": 9.0}, {"hex": "#5e3824", "pct": 7.3}]</t>
         </is>
@@ -10909,7 +11639,12 @@
           <t>ring of forms around the edge, two rectangles in the center</t>
         </is>
       </c>
-      <c r="P147" t="inlineStr">
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>Soft, sausage-like shapes in grey, ochre and brown curve around the edges of a pale canvas, while two pink rectangles float in the middle. The rounded shapes feel organic, almost like body parts or creatures, while the rectangles feel geometric and man-made. This contrast between natural and artificial forms is the heart of the work. It may be read as a playful, mysterious arrangement.</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
         <is>
           <t>[{"hex": "#a5a79f", "pct": 48.2}, {"hex": "#8d8c7f", "pct": 18.4}, {"hex": "#98772b", "pct": 14.3}, {"hex": "#535145", "pct": 10.8}, {"hex": "#9c4858", "pct": 5.6}, {"hex": "#ebeeeb", "pct": 2.7}]</t>
         </is>
@@ -10986,7 +11721,12 @@
           <t>figures on the left, grass covering the center, river to the right</t>
         </is>
       </c>
-      <c r="P148" t="inlineStr">
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>A group of people sits at a table with a patterned tablecloth in a green mountain landscape, almost swallowed by huge raised strokes of grass, while a white river rushes nearby. The thick, sculpted grass makes nature feel overwhelming and alive. Eating together outdoors is a classic subject in art, here turned wild and dramatic. It may be read as people and nature meeting, with nature in charge.</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
         <is>
           <t>[{"hex": "#578554", "pct": 20.7}, {"hex": "#3a6f39", "pct": 20.0}, {"hex": "#a5b79b", "pct": 17.1}, {"hex": "#244726", "pct": 16.0}, {"hex": "#7e9c78", "pct": 13.8}, {"hex": "#c9d4be", "pct": 12.4}]</t>
         </is>
@@ -11063,7 +11803,12 @@
           <t>arch in the center framing the figure, vertical lines throughout</t>
         </is>
       </c>
-      <c r="P149" t="inlineStr">
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>Through an arched opening we glimpse a woman's legs in a pink high-heeled shoe and white dress, while colored lines fall like threads or rain and dark hair or branches hang nearby. Seeing only part of the figure makes the scene mysterious and intimate, like a secret glimpse. The vertical colored lines add a dreamy, layered feel. It may be read as a scene about privacy, desire or memory.</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
         <is>
           <t>[{"hex": "#a6a591", "pct": 28.7}, {"hex": "#808b82", "pct": 21.1}, {"hex": "#c4c1b0", "pct": 20.1}, {"hex": "#bb8a5e", "pct": 12.0}, {"hex": "#66685b", "pct": 11.7}, {"hex": "#38342f", "pct": 6.4}]</t>
         </is>
@@ -11140,7 +11885,12 @@
           <t>strong diagonal of the carpet toward the doorway</t>
         </is>
       </c>
-      <c r="P150" t="inlineStr">
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>A room seen from above: a red carpet runs toward a dark doorway, small framed pictures lean on blue walls, and a checkerboard sits at the side. Looking down from a high angle makes the room feel tilted and unusual, like a stage set. The paintings inside the painting suggest an artist's studio or gallery. It may be read as a quiet reflection on art, space and waiting.</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
         <is>
           <t>[{"hex": "#b68f74", "pct": 32.8}, {"hex": "#b83c2f", "pct": 17.3}, {"hex": "#425f8f", "pct": 14.8}, {"hex": "#cdd3ca", "pct": 13.3}, {"hex": "#778288", "pct": 12.8}, {"hex": "#51504b", "pct": 8.9}]</t>
         </is>
@@ -11174,7 +11924,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Two green tables with small colored balls on them stand on a yellow and orange floor, seen from above at a steep angle. The walls are teal and violet. The paint is thick and loosely applied.</t>
+          <t>Two green chairs with small colored balls on their seats stand on a yellow and orange floor, seen from above at a steep angle. The walls are teal and violet. The paint is thick and loosely applied.</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -11189,7 +11939,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>["tables", "balls", "floor", "walls"]</t>
+          <t>["chairs", "balls", "floor", "walls"]</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
@@ -11214,10 +11964,15 @@
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>two tables on a diagonal in the lower half</t>
-        </is>
-      </c>
-      <c r="P151" t="inlineStr">
+          <t>two chairs on a diagonal in the lower half</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Two green chairs with small colored balls on their seats stand on a bright yellow floor, seen from a steep angle above. The tilted view and bold flat colors make an ordinary room look strange and lively. With no people present, the chairs seem to wait for someone to arrive. It may be read as a playful image of a game room or a quiet moment before action.</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
         <is>
           <t>[{"hex": "#34a181", "pct": 27.8}, {"hex": "#7d8589", "pct": 25.6}, {"hex": "#dcd053", "pct": 14.3}, {"hex": "#0e9a56", "pct": 11.2}, {"hex": "#636d4a", "pct": 10.6}, {"hex": "#cd972f", "pct": 10.4}]</t>
         </is>
@@ -11294,7 +12049,12 @@
           <t>central triangular floor with the table in the middle</t>
         </is>
       </c>
-      <c r="P152" t="inlineStr">
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>A green ping-pong table sits on a pink-purple triangular floor in front of a huge red wall, with small players at each end. The triangle of the floor pulls your eye toward the table, the center of the action. Small figures against giant color areas make the game feel tiny and playful. It may be read as a lively, humorous picture of sport and leisure.</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
         <is>
           <t>[{"hex": "#d05e51", "pct": 38.3}, {"hex": "#ab6e86", "pct": 25.8}, {"hex": "#247b5f", "pct": 11.4}, {"hex": "#dcdcd2", "pct": 10.0}, {"hex": "#5a634c", "pct": 10.0}, {"hex": "#76b3de", "pct": 4.5}]</t>
         </is>
@@ -11313,7 +12073,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>An arched composition of a man with a moustache and cap playing an accordion beside a woman in a purple dotted dress holding a red flower. Behind them are a stone gateway, old houses with balconies, a church with a dome and a café sign reading 'ART CAFE', against a gold-leaf sky. A signature and '2021' appear at the bottom.</t>
+          <t>An arched composition of a man with a moustache and cap playing an accordion beside a woman in a purple dotted dress holding a red flower. Behind them are a stone gateway, old houses with balconies, a church with a dome and a café sign reading 'ART CAFE', against a gold-leaf sky.</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -11358,10 +12118,15 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
+          <t>A man with a moustache plays an accordion beside a woman holding a red flower, in front of an old stone gate, houses with wooden balconies, a domed church and an 'ART CAFE' sign, under a gold sky. The arch shape and gold background recall religious icons, but the subject is everyday street life. Street musicians are a beloved part of many old cities. It may be read as a warm, nostalgic tribute to an old town and its music.</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
           <t>Accordion Player</t>
         </is>
       </c>
-      <c r="P153" t="inlineStr">
+      <c r="Q153" t="inlineStr">
         <is>
           <t>[{"hex": "#cfcfce", "pct": 21.7}, {"hex": "#6f6253", "pct": 20.1}, {"hex": "#88877f", "pct": 19.0}, {"hex": "#b1aa9b", "pct": 18.5}, {"hex": "#a58058", "pct": 11.2}, {"hex": "#3c3a2f", "pct": 9.4}]</t>
         </is>
@@ -11438,7 +12203,12 @@
           <t>rooster lower right, machine upper left, formulas scattered</t>
         </is>
       </c>
-      <c r="P154" t="inlineStr">
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>A large rooster stands on a blue background covered with handwritten formulas and sums like '2+2=?', while a strange flying machine carries tiny figures above. Mixing science symbols with a farm animal and a fantastical machine creates a funny, absurd scene. It may poke fun at people who overthink things, or celebrate eccentric inventors and dreamers. The handwriting feels like notes on a chalkboard.</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
         <is>
           <t>[{"hex": "#96aaba", "pct": 38.1}, {"hex": "#bac5c7", "pct": 23.2}, {"hex": "#76909e", "pct": 21.5}, {"hex": "#a99485", "pct": 11.3}, {"hex": "#705c4d", "pct": 3.9}, {"hex": "#ebca4c", "pct": 2.0}]</t>
         </is>
@@ -11502,10 +12272,15 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
+          <t>A falcon-headed god holds hands with a queen in a tall feathered crown, with hieroglyphs above them. This is painted in the style of ancient Egyptian art, where figures are shown with heads and legs in profile and shoulders facing forward. The falcon-headed god resembles Horus, a sky god linked with kingship. Painted papyrus sheets like this are popular reproductions of ancient tomb and temple art.</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
           <t>Horus and the Queen</t>
         </is>
       </c>
-      <c r="P155" t="inlineStr">
+      <c r="Q155" t="inlineStr">
         <is>
           <t>[{"hex": "#b7ae9d", "pct": 29.6}, {"hex": "#a39786", "pct": 18.1}, {"hex": "#c7c4b6", "pct": 16.8}, {"hex": "#837669", "pct": 12.6}, {"hex": "#62534c", "pct": 12.6}, {"hex": "#362c2b", "pct": 10.3}]</t>
         </is>
@@ -11569,10 +12344,15 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
+          <t>This papyrus is a chart that matches Egyptian hieroglyphs to Latin letters, with number symbols along the bottom. It shows that hieroglyphs were a real writing system, with signs for sounds and numbers. Many signs are animals, body parts or objects, like an owl, a foot or a hand. It is both decorative and educational, a popular souvenir-style reproduction.</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
           <t>Hieroglyphic Alphabet</t>
         </is>
       </c>
-      <c r="P156" t="inlineStr">
+      <c r="Q156" t="inlineStr">
         <is>
           <t>[{"hex": "#bdb19e", "pct": 27.8}, {"hex": "#d0c7b6", "pct": 22.6}, {"hex": "#a69985", "pct": 20.7}, {"hex": "#897d6a", "pct": 16.3}, {"hex": "#675b4b", "pct": 9.1}, {"hex": "#322a25", "pct": 3.6}]</t>
         </is>
@@ -11636,10 +12416,15 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
+          <t>A seated goddess with a horned sun-disc crown receives lotus flowers from a standing pharaoh, with hieroglyphs above. The horned sun-disc crown is associated with goddesses like Hathor or Isis in ancient Egyptian art. Offering scenes like this were painted in temples to show the king honoring the gods. This sheet is a modern reproduction in the traditional Egyptian style.</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
           <t>The Offering</t>
         </is>
       </c>
-      <c r="P157" t="inlineStr">
+      <c r="Q157" t="inlineStr">
         <is>
           <t>[{"hex": "#d0c2a3", "pct": 27.6}, {"hex": "#baa887", "pct": 19.7}, {"hex": "#6a503d", "pct": 15.8}, {"hex": "#392d24", "pct": 13.3}, {"hex": "#897861", "pct": 13.3}, {"hex": "#b17e44", "pct": 10.3}]</t>
         </is>
@@ -11703,10 +12488,15 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
+          <t>A man in a boat hunts birds in a papyrus marsh with a throwing stick, while a woman stands behind him and fish swim below. Marsh-hunting scenes come from ancient Egyptian tomb paintings, where they showed the good life the dead hoped to enjoy forever. The flock of colorful birds rising from the reeds makes the scene lively. This papyrus is a modern reproduction in that ancient style.</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
           <t>Hunting in the Marshes</t>
         </is>
       </c>
-      <c r="P158" t="inlineStr">
+      <c r="Q158" t="inlineStr">
         <is>
           <t>[{"hex": "#d3c5a6", "pct": 28.7}, {"hex": "#c4ac87", "pct": 18.6}, {"hex": "#9a8360", "pct": 17.7}, {"hex": "#735541", "pct": 17.4}, {"hex": "#432f28", "pct": 13.3}, {"hex": "#426691", "pct": 4.2}]</t>
         </is>
@@ -11770,10 +12560,15 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
+          <t>A large Eye of Horus is shown between a vulture with spread wings and a rearing cobra. In ancient Egyptian belief, the Eye of Horus was a powerful symbol of protection and healing, and the vulture and cobra were protective symbols of Upper and Lower Egypt. Together they form a strong protective emblem. The papyrus is a modern decorative reproduction.</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
           <t>Eye of Horus</t>
         </is>
       </c>
-      <c r="P159" t="inlineStr">
+      <c r="Q159" t="inlineStr">
         <is>
           <t>[{"hex": "#d9ccaf", "pct": 26.5}, {"hex": "#ac8e61", "pct": 17.6}, {"hex": "#8f6b4b", "pct": 16.3}, {"hex": "#cab686", "pct": 15.6}, {"hex": "#362e29", "pct": 12.9}, {"hex": "#5a4c3d", "pct": 11.2}]</t>
         </is>
@@ -11837,10 +12632,15 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
+          <t>A pharaoh draws a bow while a lion runs at his feet and a queen kneels beside him handing him an arrow, with birds flying from papyrus plants. Hunting scenes showed the king's strength and his control over nature. The queen's gesture adds a sense of partnership. This is a modern papyrus reproduction in the ancient Egyptian style.</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
           <t>The Royal Hunt</t>
         </is>
       </c>
-      <c r="P160" t="inlineStr">
+      <c r="Q160" t="inlineStr">
         <is>
           <t>[{"hex": "#8c6e4c", "pct": 20.7}, {"hex": "#a8925f", "pct": 19.8}, {"hex": "#6f4c37", "pct": 18.1}, {"hex": "#d5caae", "pct": 17.6}, {"hex": "#382f24", "pct": 12.7}, {"hex": "#c3b289", "pct": 11.1}]</t>
         </is>
@@ -11904,10 +12704,15 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
+          <t>A queen in a feathered crown gently touches or anoints a pharaoh seated on an ornate throne, while a winged vulture spreads its wings behind him. This kind of intimate royal scene is famous from ancient Egyptian art, often showing the bond between king and queen. The hieroglyphs and cartouches would name the royal couple. It is a modern papyrus reproduction in that ancient style.</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
           <t>The Anointing</t>
         </is>
       </c>
-      <c r="P161" t="inlineStr">
+      <c r="Q161" t="inlineStr">
         <is>
           <t>[{"hex": "#d4c5a9", "pct": 26.8}, {"hex": "#9b825b", "pct": 20.0}, {"hex": "#765f42", "pct": 18.0}, {"hex": "#bea679", "pct": 16.1}, {"hex": "#3e3029", "pct": 14.4}, {"hex": "#9f3c3c", "pct": 4.6}]</t>
         </is>
@@ -11971,10 +12776,15 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
+          <t>A pharaoh rides a war chariot, drawing a bow while his horse rears forward, with a vulture flying above. Battle scenes like this were carved on ancient Egyptian temple walls to show the king as a fearless hero protecting his land. The vulture is a protective symbol watching over him. This papyrus is a modern reproduction in the ancient style.</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
           <t>Pharaoh in His Chariot</t>
         </is>
       </c>
-      <c r="P162" t="inlineStr">
+      <c r="Q162" t="inlineStr">
         <is>
           <t>[{"hex": "#d1cfcd", "pct": 24.7}, {"hex": "#bfbaae", "pct": 24.6}, {"hex": "#a49d8d", "pct": 14.7}, {"hex": "#644d4a", "pct": 14.1}, {"hex": "#81786b", "pct": 12.8}, {"hex": "#363033", "pct": 9.2}]</t>
         </is>
@@ -12038,10 +12848,15 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
+          <t>Seated women in pale robes clap and play a double flute, while two dancers move on the right. Music and dance scenes come from ancient Egyptian tomb paintings of banquets, showing joy and celebration. The cones on the women's heads are a typical detail in such banquet scenes. This papyrus is a modern reproduction of that ancient art.</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
           <t>Musicians and Dancers</t>
         </is>
       </c>
-      <c r="P163" t="inlineStr">
+      <c r="Q163" t="inlineStr">
         <is>
           <t>[{"hex": "#d0c9c0", "pct": 30.4}, {"hex": "#baae9e", "pct": 20.0}, {"hex": "#9d856e", "pct": 16.6}, {"hex": "#878b9a", "pct": 11.9}, {"hex": "#6b5c54", "pct": 11.3}, {"hex": "#2e292b", "pct": 9.9}]</t>
         </is>
@@ -12105,10 +12920,15 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
+          <t>Four figures stand in a row: a goddess with a horned sun-disc crown, a pharaoh, a falcon-headed god and another pharaoh holding vessels, with hieroglyphs above. The ankh symbols they hold stand for life in ancient Egyptian belief. Scenes like this show the king being welcomed or blessed by the gods. It is a modern papyrus reproduction in the ancient style.</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
           <t>Procession of Gods</t>
         </is>
       </c>
-      <c r="P164" t="inlineStr">
+      <c r="Q164" t="inlineStr">
         <is>
           <t>[{"hex": "#bbb3a6", "pct": 25.8}, {"hex": "#d0cbc1", "pct": 24.6}, {"hex": "#9e988d", "pct": 16.0}, {"hex": "#7d7871", "pct": 12.1}, {"hex": "#58544e", "pct": 11.3}, {"hex": "#38332f", "pct": 10.1}]</t>
         </is>
@@ -12162,7 +12982,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>flat, with glare on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -12172,10 +12992,15 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
+          <t>A goddess in a red dress kneels with huge wings spread wide on both sides. Winged goddesses like this, often identified as Isis or Ma'at, were symbols of protection in ancient Egyptian art, sheltering the dead or the king under their wings. The perfectly symmetrical wings make the image calm and powerful. It is a modern papyrus reproduction.</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
           <t>The Winged Goddess</t>
         </is>
       </c>
-      <c r="P165" t="inlineStr">
+      <c r="Q165" t="inlineStr">
         <is>
           <t>[{"hex": "#b8b19f", "pct": 28.1}, {"hex": "#cdcac0", "pct": 24.5}, {"hex": "#948e80", "pct": 18.5}, {"hex": "#75695b", "pct": 16.6}, {"hex": "#453e3b", "pct": 7.8}, {"hex": "#c44e58", "pct": 4.6}]</t>
         </is>
@@ -12239,10 +13064,15 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
+          <t>A god in a white crown sits on a throne, protected by a winged goddess behind him, while a woman presents an offering table and an Eye of Horus appears nearby. The seated god resembles Osiris, the ruler of the afterlife, often shown receiving offerings. Such scenes expressed hope for protection and eternal life. It is a modern reproduction in ancient Egyptian style.</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
           <t>Offering to Osiris</t>
         </is>
       </c>
-      <c r="P166" t="inlineStr">
+      <c r="Q166" t="inlineStr">
         <is>
           <t>[{"hex": "#cdccc6", "pct": 29.5}, {"hex": "#b8b098", "pct": 23.7}, {"hex": "#958b72", "pct": 17.2}, {"hex": "#6d6054", "pct": 12.4}, {"hex": "#38363c", "pct": 11.4}, {"hex": "#be4c54", "pct": 5.8}]</t>
         </is>
@@ -12296,7 +13126,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>flat, with glare on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -12306,10 +13136,15 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
+          <t>A kneeling winged goddess faces a goddess with a horned sun-disc crown sitting on a throne, with hieroglyphs between them. The outstretched wings are a gesture of protection, and the meeting suggests a sacred ritual between divine figures. The careful symmetry and profiles are typical of ancient Egyptian art. It is a modern papyrus reproduction.</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
           <t>Two Goddesses</t>
         </is>
       </c>
-      <c r="P167" t="inlineStr">
+      <c r="Q167" t="inlineStr">
         <is>
           <t>[{"hex": "#cfcabe", "pct": 27.0}, {"hex": "#b5ae9f", "pct": 20.2}, {"hex": "#6d6452", "pct": 17.1}, {"hex": "#8c877d", "pct": 15.7}, {"hex": "#413d3a", "pct": 13.3}, {"hex": "#a68749", "pct": 6.6}]</t>
         </is>
@@ -12328,7 +13163,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>A profile bust of an Egyptian queen with a tall flat-topped dark blue crown banded in red and gold, and a broad patterned collar. The figure is drawn with simple outlines on light papyrus. Strong reflections of a window and sky cover the glass.</t>
+          <t>A profile bust of an Egyptian queen with a tall flat-topped dark blue crown banded in red and gold, and a broad patterned collar. The figure is drawn with simple outlines on light papyrus.</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -12363,7 +13198,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>flat, with strong reflections on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -12373,10 +13208,15 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
+          <t>A profile bust of a queen wears a tall, flat-topped blue crown and a broad patterned collar. Its shape strongly recalls the famous ancient Egyptian portrait of Queen Nefertiti, a symbol of beauty and elegance. The simple outlines on light papyrus focus attention on her graceful profile. It is a modern decorative reproduction.</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
           <t>Queen in Profile</t>
         </is>
       </c>
-      <c r="P168" t="inlineStr">
+      <c r="Q168" t="inlineStr">
         <is>
           <t>[{"hex": "#9f9c96", "pct": 26.5}, {"hex": "#acafac", "pct": 22.6}, {"hex": "#908578", "pct": 16.5}, {"hex": "#2f2f32", "pct": 14.2}, {"hex": "#675f58", "pct": 10.7}, {"hex": "#d3e1eb", "pct": 9.6}]</t>
         </is>
@@ -12395,7 +13235,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>An Egyptian-style papyrus scene of three female musicians: one plays a lute, one a long-necked instrument and one a harp, with a nude dancer-musician in the middle. Offering stands with vessels and grapes appear at the top. Strong reflections of windows cover the glass.</t>
+          <t>An Egyptian-style papyrus scene of three female musicians: one plays a lute, one a long-necked instrument and one a harp, with a nude dancer-musician in the middle. Offering stands with vessels and grapes appear at the top.</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -12430,7 +13270,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>flat, with strong reflections on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -12440,10 +13280,15 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
+          <t>Three women play a lute, a long-necked instrument and a harp, with a dancer-musician in the middle and offerings of food above them. Musicians like these come from ancient Egyptian tomb paintings of feasts, showing a world of pleasure and celebration. The flowing poses create a gentle rhythm across the group. It is a modern papyrus reproduction.</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
           <t>Three Musicians</t>
         </is>
       </c>
-      <c r="P169" t="inlineStr">
+      <c r="Q169" t="inlineStr">
         <is>
           <t>[{"hex": "#b8bfc0", "pct": 24.1}, {"hex": "#938377", "pct": 21.7}, {"hex": "#a5a29c", "pct": 21.1}, {"hex": "#776255", "pct": 14.5}, {"hex": "#3b3532", "pct": 9.5}, {"hex": "#e6f3fa", "pct": 9.1}]</t>
         </is>
@@ -12462,7 +13307,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>An Egyptian-style papyrus scene of two women walking hand in hand: a goddess with a horned sun-disc crown in a patterned purple and white dress holding a staff, and a queen in a tall feathered crown and pleated robe. Hieroglyphs and a cartouche are placed around them. Glare is visible on the glass.</t>
+          <t>An Egyptian-style papyrus scene of two women walking hand in hand: a goddess with a horned sun-disc crown in a patterned purple and white dress holding a staff, and a queen in a tall feathered crown and pleated robe. Hieroglyphs and a cartouche are placed around them.</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -12497,7 +13342,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>flat, with glare on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -12507,10 +13352,15 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
+          <t>A goddess with a horned sun-disc crown leads a queen by the hand, both shown in elegant profile. In ancient Egyptian art, gods taking a person by the hand often means guiding or welcoming them, for example into the afterlife. The patterned dress and tall crowns show status and divinity. It is a modern papyrus reproduction in the ancient style.</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
           <t>Goddess and Queen</t>
         </is>
       </c>
-      <c r="P170" t="inlineStr">
+      <c r="Q170" t="inlineStr">
         <is>
           <t>[{"hex": "#999894", "pct": 23.9}, {"hex": "#7e7973", "pct": 21.5}, {"hex": "#b9bcba", "pct": 20.2}, {"hex": "#2d2a2d", "pct": 16.0}, {"hex": "#5c5450", "pct": 13.8}, {"hex": "#ecf6fa", "pct": 4.6}]</t>
         </is>
@@ -12529,7 +13379,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>An Egyptian-style papyrus profile bust of a queen wearing a vulture headdress and a broad red and gold collar, with long black hair. Hieroglyphs and a cartouche frame the head, and a band of lotus motifs runs along the bottom. Reflections of a window obscure part of the face.</t>
+          <t>An Egyptian-style papyrus profile bust of a queen wearing a vulture headdress and a broad red and gold collar, with long black hair. Hieroglyphs and a cartouche frame the head, and a band of lotus motifs runs along the bottom.</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -12564,7 +13414,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>flat, with reflections on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -12574,10 +13424,15 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
+          <t>A queen in profile wears a vulture headdress and a wide red and gold collar, framed by hieroglyphs and a band of lotus flowers. The vulture crown was worn by Egyptian queens as a sign of protection and royal power, and the lotus was a symbol of rebirth. The clean outlines make the profile elegant and calm. It is a modern papyrus reproduction.</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
           <t>Queen with Vulture Crown</t>
         </is>
       </c>
-      <c r="P171" t="inlineStr">
+      <c r="Q171" t="inlineStr">
         <is>
           <t>[{"hex": "#918f87", "pct": 30.8}, {"hex": "#a8a7a0", "pct": 21.3}, {"hex": "#747069", "pct": 14.8}, {"hex": "#282123", "pct": 14.7}, {"hex": "#534a45", "pct": 12.0}, {"hex": "#deebf7", "pct": 6.4}]</t>
         </is>
@@ -12641,10 +13496,15 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
+          <t>A small white tower stands on a tiny island in the water, with a skyline of domes and minarets behind it and a rowing boat in front. The scene resembles Istanbul's famous Maiden's Tower on the Bosphorus, a landmark full of legends. Painting it almost only in black, white and grey makes it feel like an old photograph or a memory. The boat and birds add a quiet, nostalgic mood.</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
           <t>Maiden's Tower</t>
         </is>
       </c>
-      <c r="P172" t="inlineStr">
+      <c r="Q172" t="inlineStr">
         <is>
           <t>[{"hex": "#c5bdb3", "pct": 26.0}, {"hex": "#a19b94", "pct": 25.3}, {"hex": "#7e7b76", "pct": 17.7}, {"hex": "#d9d6d1", "pct": 10.7}, {"hex": "#252324", "pct": 10.4}, {"hex": "#575452", "pct": 9.9}]</t>
         </is>
@@ -12708,10 +13568,15 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
+          <t>Colorful wooden boats with tall masts crowd a calm harbor under a pastel pink and blue sky. The thick palette-knife strokes make the boats and water sparkle with texture. Harbors are a classic subject that suggest travel, work and rest at the end of the day. The soft colors give the scene a peaceful, nostalgic mood.</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
           <t>Harbor at Dusk</t>
         </is>
       </c>
-      <c r="P173" t="inlineStr">
+      <c r="Q173" t="inlineStr">
         <is>
           <t>[{"hex": "#bcb8af", "pct": 23.8}, {"hex": "#a1a09b", "pct": 22.0}, {"hex": "#808b8f", "pct": 19.5}, {"hex": "#d8d2c3", "pct": 16.0}, {"hex": "#706e67", "pct": 11.7}, {"hex": "#40403e", "pct": 7.0}]</t>
         </is>
@@ -12775,10 +13640,15 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
+          <t>A white passenger ferry cuts through choppy water toward us, with a city skyline of domes, minarets and a stone tower behind. Ferries crossing between shores are a daily part of life in waterside cities like Istanbul, which this skyline resembles. The black-and-white palette makes it feel timeless, like an old postcard. The gulls and waves give it movement and a fresh sea breeze.</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
           <t>The Ferry</t>
         </is>
       </c>
-      <c r="P174" t="inlineStr">
+      <c r="Q174" t="inlineStr">
         <is>
           <t>[{"hex": "#d4d1cb", "pct": 26.7}, {"hex": "#7a7a77", "pct": 19.4}, {"hex": "#959490", "pct": 17.7}, {"hex": "#60605e", "pct": 15.7}, {"hex": "#bab6af", "pct": 14.2}, {"hex": "#3c3b3a", "pct": 6.2}]</t>
         </is>
@@ -12842,10 +13712,15 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
+          <t>From above the rooftops, a tall round stone tower with a conical roof rises over a dense old city, with water and domed mosques behind. The tower resembles Istanbul's Galata Tower, a famous viewpoint over the city. The black, white and grey tones give the scene a nostalgic, old-photograph mood. It may be read as an affectionate portrait of a historic city.</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
           <t>The Tower over the Rooftops</t>
         </is>
       </c>
-      <c r="P175" t="inlineStr">
+      <c r="Q175" t="inlineStr">
         <is>
           <t>[{"hex": "#d1d1ce", "pct": 30.9}, {"hex": "#b5b3ad", "pct": 17.4}, {"hex": "#8c8983", "pct": 15.0}, {"hex": "#222120", "pct": 14.0}, {"hex": "#68645d", "pct": 12.0}, {"hex": "#44403c", "pct": 10.8}]</t>
         </is>
@@ -12909,10 +13784,15 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
+          <t>A mosque with a dome and a tall minaret stands by the water, with a suspension bridge behind it and pigeons in the square in front. The mix of an old mosque and a modern bridge shows a city where history and modern life meet. The tall, narrow format emphasizes the minaret and trees. Painted in black and white, the scene feels calm and nostalgic.</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
           <t>Mosque by the Bridge</t>
         </is>
       </c>
-      <c r="P176" t="inlineStr">
+      <c r="Q176" t="inlineStr">
         <is>
           <t>[{"hex": "#8f8a83", "pct": 22.1}, {"hex": "#aea79d", "pct": 20.6}, {"hex": "#c7c5c0", "pct": 16.6}, {"hex": "#6c6864", "pct": 14.4}, {"hex": "#494643", "pct": 13.7}, {"hex": "#2a2828", "pct": 12.7}]</t>
         </is>
@@ -12966,7 +13846,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>flat, with glare on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -12976,10 +13856,15 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
+          <t>A haloed saint on a white horse spears a green dragon, while a young woman stands bound to a tree. This is the famous legend of Saint George, who rescues a princess by slaying a dragon, a story about good defeating evil. The bright flat colors, large eyes and written labels are typical of Ethiopian Orthodox icons. These paintings are meant to be read as sacred stories rather than realistic scenes.</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
           <t>Saint George and the Dragon</t>
         </is>
       </c>
-      <c r="P177" t="inlineStr">
+      <c r="Q177" t="inlineStr">
         <is>
           <t>[{"hex": "#c2a53e", "pct": 22.4}, {"hex": "#876a50", "pct": 20.8}, {"hex": "#bfcbcc", "pct": 20.6}, {"hex": "#4d533a", "pct": 16.3}, {"hex": "#be887f", "pct": 11.0}, {"hex": "#8e9fa0", "pct": 9.0}]</t>
         </is>
@@ -13033,7 +13918,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>flat, with glare on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -13043,10 +13928,15 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
+          <t>The Virgin Mary in a blue mantle holds the Christ Child, with two winged angels holding swords above her. This is one of the most important images in Christian art, showing motherly love and divine protection. The large almond-shaped eyes, flat bright colors and patterned background are typical of Ethiopian Orthodox icons. The angels act as guardians around the holy pair.</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
           <t>Madonna with Angels</t>
         </is>
       </c>
-      <c r="P178" t="inlineStr">
+      <c r="Q178" t="inlineStr">
         <is>
           <t>[{"hex": "#c9a744", "pct": 24.4}, {"hex": "#5b6365", "pct": 22.5}, {"hex": "#a6826d", "pct": 18.6}, {"hex": "#6a82a9", "pct": 12.7}, {"hex": "#9d4e41", "pct": 11.3}, {"hex": "#d0cdb8", "pct": 10.5}]</t>
         </is>
@@ -13110,10 +14000,15 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
+          <t>A rider in a red cloak holds a long lance on a white horse, with an angel in the corner and writing near the top. This appears to be part of a Saint George scene, a popular subject in Ethiopian Orthodox art showing a holy warrior defeating evil. The strong outlines and flat colors make the figures clear and easy to read. The writing names the holy figures, as is typical in these icons.</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
           <t>Saint George</t>
         </is>
       </c>
-      <c r="P179" t="inlineStr">
+      <c r="Q179" t="inlineStr">
         <is>
           <t>[{"hex": "#bcae90", "pct": 26.2}, {"hex": "#7d8686", "pct": 18.9}, {"hex": "#4e5059", "pct": 14.8}, {"hex": "#794646", "pct": 13.8}, {"hex": "#a76167", "pct": 13.6}, {"hex": "#c8cbd0", "pct": 12.8}]</t>
         </is>
@@ -13177,10 +14072,15 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
+          <t>This is a painting in the Ethiopian Orthodox icon tradition showing Saint George, a Christian soldier-saint, killing a dragon from his white horse. In the legend, the dragon stands for evil and the figure in the tree is the princess he saves, so the scene is about courage and faith defeating danger. Notice the flat, bright colors and the large almond-shaped eyes: icons are not meant to look realistic, they are meant to be read like a sacred story. The writing in Ge'ez, Ethiopia's old church script, names the figures, which is typical for these icons.</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
           <t>Saint George and the Dragon</t>
         </is>
       </c>
-      <c r="P180" t="inlineStr">
+      <c r="Q180" t="inlineStr">
         <is>
           <t>[{"hex": "#c4a974", "pct": 30.0}, {"hex": "#7f6761", "pct": 23.9}, {"hex": "#3a383d", "pct": 21.5}, {"hex": "#979bb2", "pct": 11.2}, {"hex": "#d4dae0", "pct": 7.5}, {"hex": "#316cad", "pct": 5.8}]</t>
         </is>
@@ -13244,10 +14144,15 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
+          <t>The Virgin Mary sits with the Christ Child on her lap, while two angels holding swords stand behind her. The angels act as protectors, and the holy pair is shown calm and frontal, inviting prayer. Large eyes, outlined shapes and dotted patterns are typical of Ethiopian Orthodox icon painting. The red writing names the holy figures.</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
           <t>Madonna Enthroned</t>
         </is>
       </c>
-      <c r="P181" t="inlineStr">
+      <c r="Q181" t="inlineStr">
         <is>
           <t>[{"hex": "#575b5b", "pct": 24.4}, {"hex": "#383a3d", "pct": 21.2}, {"hex": "#c59d72", "pct": 20.1}, {"hex": "#985d4d", "pct": 14.2}, {"hex": "#8a8273", "pct": 12.3}, {"hex": "#cdc1a5", "pct": 7.9}]</t>
         </is>
@@ -13311,10 +14216,15 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
+          <t>Five pink and peach roses on a branch, from tight buds to fully open flowers, stand against a soft green background. Showing roses at different stages can suggest the passing of time, from youth to full bloom. Roses are a classic symbol of love and beauty. The gentle colors and careful painting give the picture a romantic, calm mood.</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
           <t>Pink Roses</t>
         </is>
       </c>
-      <c r="P182" t="inlineStr">
+      <c r="Q182" t="inlineStr">
         <is>
           <t>[{"hex": "#6b7a51", "pct": 23.6}, {"hex": "#88996f", "pct": 19.9}, {"hex": "#b5aa94", "pct": 19.4}, {"hex": "#455a49", "pct": 18.4}, {"hex": "#d2cdc0", "pct": 13.8}, {"hex": "#9e5e56", "pct": 4.9}]</t>
         </is>
@@ -13378,10 +14288,15 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
+          <t>A sunny street leads to a grand building with blue tiled domes and a decorated entrance, with a tall minaret on the left. Blue domes and tile work like this are typical of the historic cities of Central Asia along the old Silk Road. The warm sandy walls and hazy light create a feeling of heat and history. The small figures show how monumental the architecture is.</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
           <t>Old Samarkand Street</t>
         </is>
       </c>
-      <c r="P183" t="inlineStr">
+      <c r="Q183" t="inlineStr">
         <is>
           <t>[{"hex": "#cbcdbf", "pct": 26.3}, {"hex": "#9f8d7f", "pct": 22.5}, {"hex": "#b8a791", "pct": 17.5}, {"hex": "#7d716e", "pct": 16.1}, {"hex": "#9cabaf", "pct": 9.5}, {"hex": "#5e4b3e", "pct": 8.1}]</t>
         </is>
@@ -13415,7 +14330,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>A white house with small dark windows stands between two dark round trees under a deep blue night sky. The paint is extremely thick and crusty, built up in lumps. A signature and '2021' are in the lower left.</t>
+          <t>A white house with small dark windows stands between two dark round trees under a deep blue night sky. The paint is extremely thick and crusty, built up in lumps.</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -13458,7 +14373,12 @@
           <t>house in the center framed by two trees</t>
         </is>
       </c>
-      <c r="P184" t="inlineStr">
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>A small white house stands between two dark round trees under a deep blue night sky. The paint is so thick and lumpy that the picture almost becomes a relief. The bright house glows against the dark trees, giving it a mysterious, quiet feeling. It may be read as a lonely or peaceful place at night.</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
         <is>
           <t>[{"hex": "#302925", "pct": 28.9}, {"hex": "#494946", "pct": 25.1}, {"hex": "#657388", "pct": 14.4}, {"hex": "#736f4a", "pct": 12.3}, {"hex": "#aea17c", "pct": 10.1}, {"hex": "#dbcdac", "pct": 9.2}]</t>
         </is>
@@ -13477,7 +14397,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>A densely packed hillside town of small houses with red, white and yellow walls, arched windows and red striped roofs, outlined in thick black lines. A winding yellow road cuts diagonally through the houses. The work is under glass with glare.</t>
+          <t>A densely packed hillside town of small houses with red, white and yellow walls, arched windows and red striped roofs, outlined in thick black lines. A winding yellow road cuts diagonally through the houses.</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -13512,7 +14432,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>flat, with glare on glass</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -13522,10 +14442,15 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
+          <t>Small houses with colorful walls, arched windows and striped roofs crowd a hillside, with a winding yellow road running through them. The thick black outlines and bright colors give it a cheerful, naive style. Packed houses on a slope are typical of many old towns built on hills. It may be read as an affectionate picture of a lively old neighborhood.</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
           <t>Old Town Houses</t>
         </is>
       </c>
-      <c r="P185" t="inlineStr">
+      <c r="Q185" t="inlineStr">
         <is>
           <t>[{"hex": "#b2a992", "pct": 22.8}, {"hex": "#8a8579", "pct": 20.8}, {"hex": "#cccec2", "pct": 17.7}, {"hex": "#6d5d4f", "pct": 17.3}, {"hex": "#44372f", "pct": 12.5}, {"hex": "#b38645", "pct": 9.0}]</t>
         </is>
@@ -13544,7 +14469,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>A bustling Central Asian street scene with figures in turbans and long robes walking and riding donkeys toward a large arched gateway. A blue-tiled dome rises behind yellow sunlit walls, and a man sits by the roadside on the left. A signature and '2016' appear in the lower left.</t>
+          <t>A bustling Central Asian street scene with figures in turbans and long robes walking and riding donkeys toward a large arched gateway. A blue-tiled dome rises behind yellow sunlit walls, and a man sits by the roadside on the left.</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -13589,10 +14514,15 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
+          <t>People in turbans and long robes walk and ride donkeys toward a large arched gateway, with a blue-tiled dome above sunlit yellow walls. This kind of architecture recalls the old trading cities of Central Asia along the Silk Road. The strong sunlight and blue shadows make the street feel hot and busy. It may be read as a lively picture of an old bazaar street.</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
           <t>Bazaar Street</t>
         </is>
       </c>
-      <c r="P186" t="inlineStr">
+      <c r="Q186" t="inlineStr">
         <is>
           <t>[{"hex": "#bdc4c2", "pct": 28.5}, {"hex": "#c8a659", "pct": 18.6}, {"hex": "#93968d", "pct": 16.9}, {"hex": "#717271", "pct": 15.7}, {"hex": "#947a4f", "pct": 10.9}, {"hex": "#57453a", "pct": 9.4}]</t>
         </is>
@@ -13656,10 +14586,15 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
+          <t>Two decorated white elephants raise their trunks toward each other in the center, surrounded by twelve circles with animals and figures like a fish, a bull, a ram and an archer. These twelve signs resemble the zodiac, used in astrology to represent times of the year and personality types. The rich gold and floral decoration is typical of Southeast Asian decorative art. It may be read as a symbolic map of the year and fortune.</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
           <t>Zodiac Wheel</t>
         </is>
       </c>
-      <c r="P187" t="inlineStr">
+      <c r="Q187" t="inlineStr">
         <is>
           <t>[{"hex": "#918162", "pct": 34.7}, {"hex": "#66644f", "pct": 24.0}, {"hex": "#b0a283", "pct": 23.1}, {"hex": "#33342f", "pct": 7.2}, {"hex": "#ad5743", "pct": 6.7}, {"hex": "#d2d1c4", "pct": 4.2}]</t>
         </is>
@@ -13723,10 +14658,15 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
+          <t>White and terracotta temples and pagodas rise among dark trees under a glowing pink-orange sky with a pale moon or sun. The glittering surface is made with sand, a special technique that catches the light. Fields of ancient temples like this are found in parts of Southeast Asia and are places of pilgrimage. The dusk light gives the scene a peaceful, spiritual mood.</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
           <t>Temples at Dusk</t>
         </is>
       </c>
-      <c r="P188" t="inlineStr">
+      <c r="Q188" t="inlineStr">
         <is>
           <t>[{"hex": "#c0a16f", "pct": 26.1}, {"hex": "#595d54", "pct": 21.9}, {"hex": "#ac8561", "pct": 21.0}, {"hex": "#787261", "pct": 18.2}, {"hex": "#cdc9c1", "pct": 7.6}, {"hex": "#969d95", "pct": 5.1}]</t>
         </is>
@@ -13790,10 +14730,15 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
+          <t>Two tall tree trunks stand on the right of a sunny garden, with green foliage above and a low stone wall or bench below. Bright yellow-green light and loose brushwork give the scene a warm summer feeling. Painting outdoors to capture light quickly is an impressionist approach. It may be read as a peaceful moment in a park on a sunny day.</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
           <t>In the Garden</t>
         </is>
       </c>
-      <c r="P189" t="inlineStr">
+      <c r="Q189" t="inlineStr">
         <is>
           <t>[{"hex": "#827937", "pct": 29.9}, {"hex": "#a08418", "pct": 24.5}, {"hex": "#979665", "pct": 15.5}, {"hex": "#cab21a", "pct": 12.0}, {"hex": "#9badac", "pct": 10.8}, {"hex": "#ecd263", "pct": 7.3}]</t>
         </is>
@@ -13857,10 +14802,15 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
+          <t>Stylized figures with mask-like faces, beaded necklaces and striped clothes are packed tightly together, outlined in thick black lines and bright flat colors. The style mixes cubist fragmentation with African mask traditions. The crowded, interlocking shapes create a strong sense of rhythm, music and dance. It may be read as a celebration or festival full of energy.</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
           <t>Festival</t>
         </is>
       </c>
-      <c r="P190" t="inlineStr">
+      <c r="Q190" t="inlineStr">
         <is>
           <t>[{"hex": "#2b2d26", "pct": 28.6}, {"hex": "#7b5039", "pct": 19.9}, {"hex": "#c0a551", "pct": 19.7}, {"hex": "#555c71", "pct": 11.5}, {"hex": "#97aa9b", "pct": 10.6}, {"hex": "#cfd6c6", "pct": 9.7}]</t>
         </is>
@@ -13879,7 +14829,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>An abstracted market or riverside scene in palette-knife strokes, with figures in white conical hats carrying baskets on shoulder poles. Reds, greens, blues and blacks are set against a bright yellow ground. A signature appears in the lower left.</t>
+          <t>An abstracted market or riverside scene in palette-knife strokes, with figures in white conical hats carrying baskets on shoulder poles. Reds, greens, blues and blacks are set against a bright yellow ground.</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -13924,10 +14874,15 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
+          <t>Figures in white conical hats carry baskets on shoulder poles, painted with bold palette-knife strokes on a bright yellow background. Conical hats and shoulder poles are typical of markets and river life in parts of Southeast Asia. The abstract style captures movement and color more than details. It may be read as a busy, sunny market morning.</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
           <t>Market Morning</t>
         </is>
       </c>
-      <c r="P191" t="inlineStr">
+      <c r="Q191" t="inlineStr">
         <is>
           <t>[{"hex": "#c0aa3d", "pct": 27.2}, {"hex": "#9b6c35", "pct": 18.1}, {"hex": "#653d26", "pct": 17.0}, {"hex": "#1e1e17", "pct": 15.9}, {"hex": "#c2b9a3", "pct": 14.7}, {"hex": "#626b77", "pct": 7.2}]</t>
         </is>
@@ -13946,7 +14901,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>An empty room seen in perspective with mustard-yellow walls and floor, and a window or painting opening onto a green landscape and blue sky at the back. Two dark figures embrace in the middle of the room, and two white dandelion-like circles sit on the floor. Yellow and dark paint is splattered across; a Georgian signature and '2019' appear at the lower right.</t>
+          <t>An empty room seen in perspective with mustard-yellow walls and floor, and a window or painting opening onto a green landscape and blue sky at the back. Two dark figures embrace in the middle of the room, and two white dandelion-like circles sit on the floor. Yellow and dark paint is splattered across.</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -13961,7 +14916,7 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>["room", "window", "landscape", "figures", "dandelions", "signature"]</t>
+          <t>["room", "window", "landscape", "figures", "dandelions"]</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -13989,7 +14944,12 @@
           <t>one-point perspective room, figures center, window behind</t>
         </is>
       </c>
-      <c r="P192" t="inlineStr">
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>An empty mustard-yellow room opens onto a green landscape through a window at the back, while two dark figures embrace in the middle. Two white dandelion-like circles sit on the floor, and paint is splattered across the surface. The empty room makes the embrace feel private and important. It may be read as a picture of love, longing or a memory, with the window suggesting hope or the world outside.</t>
+        </is>
+      </c>
+      <c r="Q192" t="inlineStr">
         <is>
           <t>[{"hex": "#c59933", "pct": 29.8}, {"hex": "#917c37", "pct": 24.1}, {"hex": "#5c4c32", "pct": 16.2}, {"hex": "#9dafd2", "pct": 14.3}, {"hex": "#e0c44b", "pct": 8.8}, {"hex": "#8c8d83", "pct": 6.7}]</t>
         </is>
@@ -14053,10 +15013,15 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
+          <t>Five tall women in red dresses walk in a rhythmic line, two carrying pots on their heads, against a huge glowing sun. The red figures against the yellow and white sun create a strong, warm contrast. Their crossing legs make the line feel like a dance. It may be read as a celebration of women, daily work and the beauty of the evening.</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
           <t>Walking Home</t>
         </is>
       </c>
-      <c r="P193" t="inlineStr">
+      <c r="Q193" t="inlineStr">
         <is>
           <t>[{"hex": "#c21e24", "pct": 28.5}, {"hex": "#852829", "pct": 24.8}, {"hex": "#deb431", "pct": 16.1}, {"hex": "#d7702a", "pct": 12.8}, {"hex": "#342729", "pct": 12.7}, {"hex": "#d0d8c5", "pct": 5.1}]</t>
         </is>
@@ -14120,10 +15085,15 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
+          <t>A herd of dark cattle is driven by herders in red cloaks under a large flat-topped acacia tree, with a snow-capped mountain in the distance. Acacia trees, savanna grass and red cloaks recall the landscapes and herding traditions of East Africa. The wide panoramic format makes the land feel vast. It may be read as a peaceful picture of pastoral life.</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
           <t>Herders below Kilimanjaro</t>
         </is>
       </c>
-      <c r="P194" t="inlineStr">
+      <c r="Q194" t="inlineStr">
         <is>
           <t>[{"hex": "#9c9d9a", "pct": 25.8}, {"hex": "#b6b6b0", "pct": 22.8}, {"hex": "#705735", "pct": 15.4}, {"hex": "#927e4d", "pct": 13.7}, {"hex": "#757d8a", "pct": 12.4}, {"hex": "#473022", "pct": 10.0}]</t>
         </is>
@@ -14187,10 +15157,15 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
+          <t>A long, panoramic night scene shows many small boats on deep blue water, with stilt houses on both sides and a bright reflection of light in the center. The glowing reflection pulls your eye to the middle of the picture. Fishing boats and stilt houses show a life closely connected to the water. The dark blues give the scene a calm, magical night atmosphere.</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
           <t>Night on the Lake</t>
         </is>
       </c>
-      <c r="P195" t="inlineStr">
+      <c r="Q195" t="inlineStr">
         <is>
           <t>[{"hex": "#383c53", "pct": 26.1}, {"hex": "#1f212c", "pct": 26.1}, {"hex": "#505975", "pct": 21.1}, {"hex": "#7e8287", "pct": 12.3}, {"hex": "#b3b2ab", "pct": 7.5}, {"hex": "#655c4d", "pct": 6.9}]</t>
         </is>
@@ -14254,10 +15229,15 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
+          <t>Seven slender women in bright wraps walk away from us, each balancing a large white pot on her head, with reflections below them on blue ground. Carrying water in pots is a daily task in many rural communities. The quick outlines and reflections make the figures feel graceful and moving. It may be read as a tribute to women's strength and everyday work.</t>
+        </is>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
           <t>Water Carriers</t>
         </is>
       </c>
-      <c r="P196" t="inlineStr">
+      <c r="Q196" t="inlineStr">
         <is>
           <t>[{"hex": "#799a9d", "pct": 28.7}, {"hex": "#65868d", "pct": 28.5}, {"hex": "#4c6f77", "pct": 14.9}, {"hex": "#cb8b4c", "pct": 11.4}, {"hex": "#7b5f3f", "pct": 8.9}, {"hex": "#dccd9c", "pct": 7.5}]</t>
         </is>

</xml_diff>